<commit_message>
Atualiza dados — extração 05/10/2026 13:57 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -12968,7 +12968,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46300.347258368056</v>
+        <v>46300.581690150466</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -42820,7 +42820,7 @@
         <v>24000</v>
       </c>
       <c r="O569" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P569" s="0" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 06/10/2026 08:27 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -12968,7 +12968,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46300.581690150466</v>
+        <v>46301.352679270836</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -26152,7 +26152,7 @@
         <v>2</v>
       </c>
       <c r="O245" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P245" s="0" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 06/10/2026 14:52 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4261" uniqueCount="4261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4265" uniqueCount="4265">
   <si>
     <t>Geração:</t>
   </si>
@@ -12795,6 +12795,18 @@
   </si>
   <si>
     <t>VALTONIO</t>
+  </si>
+  <si>
+    <t>RXU3A18</t>
+  </si>
+  <si>
+    <t>M.BENZ/ATEGO 2426</t>
+  </si>
+  <si>
+    <t>9BM958164NB272614</t>
+  </si>
+  <si>
+    <t>01327843274</t>
   </si>
 </sst>
 </file>
@@ -12957,7 +12969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W968"/>
+  <dimension ref="A1:W969"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -12968,7 +12980,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46301.352679270836</v>
+        <v>46301.61944785879</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -62204,6 +62216,50 @@
       </c>
       <c r="R968" s="0" t="s">
         <v>4260</v>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" s="0" t="s">
+        <v>2719</v>
+      </c>
+      <c r="B969" s="10">
+        <v>46301.476280462964</v>
+      </c>
+      <c r="C969" s="0" t="s">
+        <v>2720</v>
+      </c>
+      <c r="D969" s="0" t="s">
+        <v>4261</v>
+      </c>
+      <c r="E969" s="0" t="s">
+        <v>4262</v>
+      </c>
+      <c r="F969" s="0" t="s">
+        <v>4262</v>
+      </c>
+      <c r="G969" s="0" t="s">
+        <v>2720</v>
+      </c>
+      <c r="H969" s="0" t="s">
+        <v>4263</v>
+      </c>
+      <c r="I969" s="0" t="s">
+        <v>4264</v>
+      </c>
+      <c r="J969" s="0" t="s">
+        <v>1152</v>
+      </c>
+      <c r="K969" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="L969" s="0" t="s">
+        <v>3468</v>
+      </c>
+      <c r="O969" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="R969" s="0" t="s">
+        <v>4086</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados — extração 08/10/2026 08:49 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -12980,7 +12980,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46302.352964432874</v>
+        <v>46303.36773337963</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -60890,7 +60890,7 @@
         <v>273</v>
       </c>
       <c r="O940" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P940" s="0" t="s">
         <v>3634</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 08/10/2026 15:10 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4265" uniqueCount="4265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4273" uniqueCount="4273">
   <si>
     <t>Geração:</t>
   </si>
@@ -11111,6 +11111,12 @@
     <t>ANTONIO RODRIGUES SOUSA</t>
   </si>
   <si>
+    <t>KEA6J64</t>
+  </si>
+  <si>
+    <t>MBQ6J91</t>
+  </si>
+  <si>
     <t>CD TRUCK</t>
   </si>
   <si>
@@ -12807,6 +12813,24 @@
   </si>
   <si>
     <t>01327843274</t>
+  </si>
+  <si>
+    <t>RANDON SR FG</t>
+  </si>
+  <si>
+    <t>9ADF1363YYS152858</t>
+  </si>
+  <si>
+    <t>00734741464</t>
+  </si>
+  <si>
+    <t>REB/FACCHINI-IR RER FR</t>
+  </si>
+  <si>
+    <t>9EL11FR031V005201</t>
+  </si>
+  <si>
+    <t>00753284812</t>
   </si>
 </sst>
 </file>
@@ -12969,7 +12993,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W969"/>
+  <dimension ref="A1:W971"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -12980,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46303.36773337963</v>
+        <v>46303.63243648148</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -55507,10 +55531,16 @@
       <c r="R826" s="0" t="s">
         <v>3698</v>
       </c>
+      <c r="S826" s="0" t="s">
+        <v>3699</v>
+      </c>
+      <c r="T826" s="0" t="s">
+        <v>3700</v>
+      </c>
     </row>
     <row r="827">
       <c r="A827" s="0" t="s">
-        <v>3699</v>
+        <v>3701</v>
       </c>
       <c r="B827" s="10">
         <v>46037.467388136574</v>
@@ -55519,7 +55549,7 @@
         <v>3686</v>
       </c>
       <c r="D827" s="0" t="s">
-        <v>3700</v>
+        <v>3702</v>
       </c>
       <c r="E827" s="0" t="s">
         <v>196</v>
@@ -55531,10 +55561,10 @@
         <v>3689</v>
       </c>
       <c r="H827" s="0" t="s">
-        <v>3701</v>
+        <v>3703</v>
       </c>
       <c r="I827" s="0" t="s">
-        <v>3702</v>
+        <v>3704</v>
       </c>
       <c r="J827" s="0" t="s">
         <v>209</v>
@@ -55558,7 +55588,7 @@
         <v>52</v>
       </c>
       <c r="R827" s="0" t="s">
-        <v>3703</v>
+        <v>3705</v>
       </c>
     </row>
     <row r="828">
@@ -55572,22 +55602,22 @@
         <v>3686</v>
       </c>
       <c r="D828" s="0" t="s">
-        <v>3704</v>
+        <v>3706</v>
       </c>
       <c r="E828" s="0" t="s">
-        <v>3705</v>
+        <v>3707</v>
       </c>
       <c r="F828" s="0" t="s">
-        <v>3706</v>
+        <v>3708</v>
       </c>
       <c r="G828" s="0" t="s">
         <v>3689</v>
       </c>
       <c r="H828" s="0" t="s">
-        <v>3707</v>
+        <v>3709</v>
       </c>
       <c r="I828" s="0" t="s">
-        <v>3708</v>
+        <v>3710</v>
       </c>
       <c r="J828" s="0" t="s">
         <v>506</v>
@@ -55596,7 +55626,13 @@
         <v>38</v>
       </c>
       <c r="P828" s="0" t="s">
-        <v>3705</v>
+        <v>3707</v>
+      </c>
+      <c r="S828" s="0" t="s">
+        <v>3699</v>
+      </c>
+      <c r="T828" s="0" t="s">
+        <v>3700</v>
       </c>
     </row>
     <row r="829">
@@ -55610,25 +55646,25 @@
         <v>128</v>
       </c>
       <c r="D829" s="0" t="s">
-        <v>3709</v>
+        <v>3711</v>
       </c>
       <c r="E829" s="0" t="s">
-        <v>3710</v>
+        <v>3712</v>
       </c>
       <c r="F829" s="0" t="s">
-        <v>3710</v>
+        <v>3712</v>
       </c>
       <c r="G829" s="0" t="s">
         <v>1887</v>
       </c>
       <c r="H829" s="0" t="s">
-        <v>3711</v>
+        <v>3713</v>
       </c>
       <c r="I829" s="0" t="s">
-        <v>3712</v>
+        <v>3714</v>
       </c>
       <c r="J829" s="0" t="s">
-        <v>3713</v>
+        <v>3715</v>
       </c>
       <c r="K829" s="0" t="s">
         <v>36</v>
@@ -55643,7 +55679,7 @@
         <v>512</v>
       </c>
       <c r="R829" s="0" t="s">
-        <v>3714</v>
+        <v>3716</v>
       </c>
       <c r="S829" s="0" t="s">
         <v>1905</v>
@@ -55660,25 +55696,25 @@
         <v>2720</v>
       </c>
       <c r="D830" s="0" t="s">
-        <v>3715</v>
+        <v>3717</v>
       </c>
       <c r="E830" s="0" t="s">
         <v>781</v>
       </c>
       <c r="F830" s="0" t="s">
-        <v>3716</v>
+        <v>3718</v>
       </c>
       <c r="G830" s="0" t="s">
         <v>2720</v>
       </c>
       <c r="H830" s="0" t="s">
-        <v>3717</v>
+        <v>3719</v>
       </c>
       <c r="I830" s="0" t="s">
-        <v>3718</v>
+        <v>3720</v>
       </c>
       <c r="J830" s="0" t="s">
-        <v>3719</v>
+        <v>3721</v>
       </c>
       <c r="K830" s="0" t="s">
         <v>2230</v>
@@ -55701,25 +55737,25 @@
         <v>2720</v>
       </c>
       <c r="D831" s="0" t="s">
-        <v>3720</v>
+        <v>3722</v>
       </c>
       <c r="E831" s="0" t="s">
         <v>781</v>
       </c>
       <c r="F831" s="0" t="s">
-        <v>3721</v>
+        <v>3723</v>
       </c>
       <c r="G831" s="0" t="s">
         <v>2720</v>
       </c>
       <c r="H831" s="0" t="s">
-        <v>3722</v>
+        <v>3724</v>
       </c>
       <c r="I831" s="0" t="s">
-        <v>3723</v>
+        <v>3725</v>
       </c>
       <c r="J831" s="0" t="s">
-        <v>3719</v>
+        <v>3721</v>
       </c>
       <c r="K831" s="0" t="s">
         <v>2230</v>
@@ -55742,7 +55778,7 @@
         <v>28</v>
       </c>
       <c r="D832" s="0" t="s">
-        <v>3724</v>
+        <v>3726</v>
       </c>
       <c r="E832" s="0" t="s">
         <v>60</v>
@@ -55754,10 +55790,10 @@
         <v>147</v>
       </c>
       <c r="H832" s="0" t="s">
-        <v>3725</v>
+        <v>3727</v>
       </c>
       <c r="I832" s="0" t="s">
-        <v>3726</v>
+        <v>3728</v>
       </c>
       <c r="J832" s="0" t="s">
         <v>1151</v>
@@ -55775,7 +55811,7 @@
         <v>176</v>
       </c>
       <c r="R832" s="0" t="s">
-        <v>3727</v>
+        <v>3729</v>
       </c>
       <c r="S832" s="0" t="s">
         <v>182</v>
@@ -55804,10 +55840,10 @@
         <v>147</v>
       </c>
       <c r="H833" s="0" t="s">
-        <v>3728</v>
+        <v>3730</v>
       </c>
       <c r="I833" s="0" t="s">
-        <v>3729</v>
+        <v>3731</v>
       </c>
       <c r="J833" s="0" t="s">
         <v>186</v>
@@ -55836,7 +55872,7 @@
         <v>91</v>
       </c>
       <c r="D834" s="0" t="s">
-        <v>3730</v>
+        <v>3732</v>
       </c>
       <c r="E834" s="0" t="s">
         <v>788</v>
@@ -55848,10 +55884,10 @@
         <v>1138</v>
       </c>
       <c r="H834" s="0" t="s">
-        <v>3731</v>
+        <v>3733</v>
       </c>
       <c r="I834" s="0" t="s">
-        <v>3732</v>
+        <v>3734</v>
       </c>
       <c r="J834" s="0" t="s">
         <v>160</v>
@@ -55877,7 +55913,7 @@
         <v>91</v>
       </c>
       <c r="D835" s="0" t="s">
-        <v>3733</v>
+        <v>3735</v>
       </c>
       <c r="E835" s="0" t="s">
         <v>788</v>
@@ -55889,10 +55925,10 @@
         <v>1138</v>
       </c>
       <c r="H835" s="0" t="s">
-        <v>3734</v>
+        <v>3736</v>
       </c>
       <c r="I835" s="0" t="s">
-        <v>3735</v>
+        <v>3737</v>
       </c>
       <c r="J835" s="0" t="s">
         <v>160</v>
@@ -55915,25 +55951,25 @@
         <v>46104.56253545139</v>
       </c>
       <c r="C836" s="0" t="s">
-        <v>3736</v>
+        <v>3738</v>
       </c>
       <c r="D836" s="0" t="s">
-        <v>3737</v>
+        <v>3739</v>
       </c>
       <c r="E836" s="0" t="s">
         <v>165</v>
       </c>
       <c r="F836" s="0" t="s">
-        <v>3738</v>
+        <v>3740</v>
       </c>
       <c r="G836" s="0" t="s">
-        <v>3739</v>
+        <v>3741</v>
       </c>
       <c r="H836" s="0" t="s">
-        <v>3740</v>
+        <v>3742</v>
       </c>
       <c r="I836" s="0" t="s">
-        <v>3741</v>
+        <v>3743</v>
       </c>
       <c r="J836" s="0" t="s">
         <v>1536</v>
@@ -55948,7 +55984,7 @@
         <v>38</v>
       </c>
       <c r="V836" s="0" t="s">
-        <v>3742</v>
+        <v>3744</v>
       </c>
     </row>
     <row r="837">
@@ -55974,10 +56010,10 @@
         <v>2741</v>
       </c>
       <c r="H837" s="0" t="s">
-        <v>3743</v>
+        <v>3745</v>
       </c>
       <c r="I837" s="0" t="s">
-        <v>3744</v>
+        <v>3746</v>
       </c>
       <c r="J837" s="0" t="s">
         <v>2905</v>
@@ -56009,7 +56045,7 @@
         <v>2738</v>
       </c>
       <c r="D838" s="0" t="s">
-        <v>3745</v>
+        <v>3747</v>
       </c>
       <c r="E838" s="0" t="s">
         <v>30</v>
@@ -56021,10 +56057,10 @@
         <v>2741</v>
       </c>
       <c r="H838" s="0" t="s">
-        <v>3746</v>
+        <v>3748</v>
       </c>
       <c r="I838" s="0" t="s">
-        <v>3747</v>
+        <v>3749</v>
       </c>
       <c r="J838" s="0" t="s">
         <v>3089</v>
@@ -56059,7 +56095,7 @@
         <v>91</v>
       </c>
       <c r="D839" s="0" t="s">
-        <v>3748</v>
+        <v>3750</v>
       </c>
       <c r="E839" s="0" t="s">
         <v>30</v>
@@ -56071,10 +56107,10 @@
         <v>1138</v>
       </c>
       <c r="H839" s="0" t="s">
-        <v>3749</v>
+        <v>3751</v>
       </c>
       <c r="I839" s="0" t="s">
-        <v>3750</v>
+        <v>3752</v>
       </c>
       <c r="J839" s="0" t="s">
         <v>506</v>
@@ -56092,7 +56128,7 @@
         <v>3635</v>
       </c>
       <c r="S839" s="0" t="s">
-        <v>3730</v>
+        <v>3732</v>
       </c>
     </row>
     <row r="840">
@@ -56118,10 +56154,10 @@
         <v>2741</v>
       </c>
       <c r="H840" s="0" t="s">
-        <v>3751</v>
+        <v>3753</v>
       </c>
       <c r="I840" s="0" t="s">
-        <v>3752</v>
+        <v>3754</v>
       </c>
       <c r="J840" s="0" t="s">
         <v>2905</v>
@@ -56153,7 +56189,7 @@
         <v>28</v>
       </c>
       <c r="D841" s="0" t="s">
-        <v>3753</v>
+        <v>3755</v>
       </c>
       <c r="E841" s="0" t="s">
         <v>60</v>
@@ -56165,10 +56201,10 @@
         <v>147</v>
       </c>
       <c r="H841" s="0" t="s">
-        <v>3754</v>
+        <v>3756</v>
       </c>
       <c r="I841" s="0" t="s">
-        <v>3755</v>
+        <v>3757</v>
       </c>
       <c r="J841" s="0" t="s">
         <v>169</v>
@@ -56203,7 +56239,7 @@
         <v>28</v>
       </c>
       <c r="D842" s="0" t="s">
-        <v>3756</v>
+        <v>3758</v>
       </c>
       <c r="E842" s="0" t="s">
         <v>60</v>
@@ -56215,10 +56251,10 @@
         <v>147</v>
       </c>
       <c r="H842" s="0" t="s">
-        <v>3757</v>
+        <v>3759</v>
       </c>
       <c r="I842" s="0" t="s">
-        <v>3758</v>
+        <v>3760</v>
       </c>
       <c r="J842" s="0" t="s">
         <v>1536</v>
@@ -56265,10 +56301,10 @@
         <v>147</v>
       </c>
       <c r="H843" s="0" t="s">
-        <v>3759</v>
+        <v>3761</v>
       </c>
       <c r="I843" s="0" t="s">
-        <v>3760</v>
+        <v>3762</v>
       </c>
       <c r="J843" s="0" t="s">
         <v>160</v>
@@ -56277,7 +56313,7 @@
         <v>161</v>
       </c>
       <c r="L843" s="0" t="s">
-        <v>3761</v>
+        <v>3763</v>
       </c>
       <c r="O843" s="0" t="s">
         <v>38</v>
@@ -56297,22 +56333,22 @@
         <v>128</v>
       </c>
       <c r="D844" s="0" t="s">
-        <v>3762</v>
+        <v>3764</v>
       </c>
       <c r="E844" s="0" t="s">
-        <v>3763</v>
+        <v>3765</v>
       </c>
       <c r="F844" s="0" t="s">
-        <v>3763</v>
+        <v>3765</v>
       </c>
       <c r="G844" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H844" s="0" t="s">
-        <v>3764</v>
+        <v>3766</v>
       </c>
       <c r="I844" s="0" t="s">
-        <v>3765</v>
+        <v>3767</v>
       </c>
       <c r="J844" s="0" t="s">
         <v>669</v>
@@ -56321,19 +56357,19 @@
         <v>36</v>
       </c>
       <c r="L844" s="0" t="s">
-        <v>3766</v>
+        <v>3768</v>
       </c>
       <c r="O844" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P844" s="0" t="s">
-        <v>3767</v>
+        <v>3769</v>
       </c>
       <c r="R844" s="0" t="s">
         <v>2882</v>
       </c>
       <c r="S844" s="0" t="s">
-        <v>3768</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="845">
@@ -56347,22 +56383,22 @@
         <v>128</v>
       </c>
       <c r="D845" s="0" t="s">
-        <v>3768</v>
+        <v>3770</v>
       </c>
       <c r="E845" s="0" t="s">
-        <v>3769</v>
+        <v>3771</v>
       </c>
       <c r="F845" s="0" t="s">
-        <v>3769</v>
+        <v>3771</v>
       </c>
       <c r="G845" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H845" s="0" t="s">
-        <v>3770</v>
+        <v>3772</v>
       </c>
       <c r="I845" s="0" t="s">
-        <v>3771</v>
+        <v>3773</v>
       </c>
       <c r="J845" s="0" t="s">
         <v>134</v>
@@ -56371,13 +56407,13 @@
         <v>161</v>
       </c>
       <c r="L845" s="0" t="s">
-        <v>3766</v>
+        <v>3768</v>
       </c>
       <c r="O845" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P845" s="0" t="s">
-        <v>3767</v>
+        <v>3769</v>
       </c>
       <c r="R845" s="0" t="s">
         <v>2882</v>
@@ -56394,7 +56430,7 @@
         <v>28</v>
       </c>
       <c r="D846" s="0" t="s">
-        <v>3772</v>
+        <v>3774</v>
       </c>
       <c r="E846" s="0" t="s">
         <v>196</v>
@@ -56406,10 +56442,10 @@
         <v>32</v>
       </c>
       <c r="H846" s="0" t="s">
-        <v>3773</v>
+        <v>3775</v>
       </c>
       <c r="I846" s="0" t="s">
-        <v>3774</v>
+        <v>3776</v>
       </c>
       <c r="J846" s="0" t="s">
         <v>403</v>
@@ -56418,16 +56454,16 @@
         <v>201</v>
       </c>
       <c r="L846" s="0" t="s">
-        <v>3775</v>
+        <v>3777</v>
       </c>
       <c r="O846" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P846" s="0" t="s">
-        <v>3776</v>
+        <v>3778</v>
       </c>
       <c r="R846" s="0" t="s">
-        <v>3777</v>
+        <v>3779</v>
       </c>
     </row>
     <row r="847">
@@ -56441,22 +56477,22 @@
         <v>28</v>
       </c>
       <c r="D847" s="0" t="s">
-        <v>3778</v>
+        <v>3780</v>
       </c>
       <c r="E847" s="0" t="s">
         <v>76</v>
       </c>
       <c r="F847" s="0" t="s">
-        <v>3779</v>
+        <v>3781</v>
       </c>
       <c r="G847" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H847" s="0" t="s">
-        <v>3780</v>
+        <v>3782</v>
       </c>
       <c r="I847" s="0" t="s">
-        <v>3781</v>
+        <v>3783</v>
       </c>
       <c r="J847" s="0" t="s">
         <v>1370</v>
@@ -56471,10 +56507,10 @@
         <v>51</v>
       </c>
       <c r="P847" s="0" t="s">
-        <v>3782</v>
+        <v>3784</v>
       </c>
       <c r="R847" s="0" t="s">
-        <v>3783</v>
+        <v>3785</v>
       </c>
     </row>
     <row r="848">
@@ -56488,7 +56524,7 @@
         <v>28</v>
       </c>
       <c r="D848" s="0" t="s">
-        <v>3784</v>
+        <v>3786</v>
       </c>
       <c r="E848" s="0" t="s">
         <v>60</v>
@@ -56500,10 +56536,10 @@
         <v>32</v>
       </c>
       <c r="H848" s="0" t="s">
-        <v>3785</v>
+        <v>3787</v>
       </c>
       <c r="I848" s="0" t="s">
-        <v>3786</v>
+        <v>3788</v>
       </c>
       <c r="J848" s="0" t="s">
         <v>396</v>
@@ -56512,22 +56548,22 @@
         <v>36</v>
       </c>
       <c r="L848" s="0" t="s">
-        <v>3787</v>
+        <v>3789</v>
       </c>
       <c r="O848" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P848" s="0" t="s">
-        <v>3788</v>
+        <v>3790</v>
       </c>
       <c r="R848" s="0" t="s">
         <v>2866</v>
       </c>
       <c r="S848" s="0" t="s">
-        <v>3789</v>
+        <v>3791</v>
       </c>
       <c r="T848" s="0" t="s">
-        <v>3790</v>
+        <v>3792</v>
       </c>
     </row>
     <row r="849">
@@ -56541,7 +56577,7 @@
         <v>28</v>
       </c>
       <c r="D849" s="0" t="s">
-        <v>3791</v>
+        <v>3793</v>
       </c>
       <c r="E849" s="0" t="s">
         <v>104</v>
@@ -56553,10 +56589,10 @@
         <v>32</v>
       </c>
       <c r="H849" s="0" t="s">
-        <v>3792</v>
+        <v>3794</v>
       </c>
       <c r="I849" s="0" t="s">
-        <v>3793</v>
+        <v>3795</v>
       </c>
       <c r="J849" s="0" t="s">
         <v>280</v>
@@ -56588,22 +56624,22 @@
         <v>2738</v>
       </c>
       <c r="D850" s="0" t="s">
-        <v>3794</v>
+        <v>3796</v>
       </c>
       <c r="E850" s="0" t="s">
         <v>60</v>
       </c>
       <c r="F850" s="0" t="s">
-        <v>3795</v>
+        <v>3797</v>
       </c>
       <c r="G850" s="0" t="s">
         <v>2741</v>
       </c>
       <c r="H850" s="0" t="s">
-        <v>3796</v>
+        <v>3798</v>
       </c>
       <c r="I850" s="0" t="s">
-        <v>3797</v>
+        <v>3799</v>
       </c>
       <c r="J850" s="0" t="s">
         <v>1830</v>
@@ -56638,7 +56674,7 @@
         <v>28</v>
       </c>
       <c r="D851" s="0" t="s">
-        <v>3798</v>
+        <v>3800</v>
       </c>
       <c r="E851" s="0" t="s">
         <v>60</v>
@@ -56650,10 +56686,10 @@
         <v>32</v>
       </c>
       <c r="H851" s="0" t="s">
-        <v>3799</v>
+        <v>3801</v>
       </c>
       <c r="I851" s="0" t="s">
-        <v>3800</v>
+        <v>3802</v>
       </c>
       <c r="J851" s="0" t="s">
         <v>454</v>
@@ -56668,13 +56704,13 @@
         <v>38</v>
       </c>
       <c r="P851" s="0" t="s">
-        <v>3801</v>
+        <v>3803</v>
       </c>
       <c r="R851" s="0" t="s">
         <v>1502</v>
       </c>
       <c r="S851" s="0" t="s">
-        <v>3802</v>
+        <v>3804</v>
       </c>
     </row>
     <row r="852">
@@ -56688,7 +56724,7 @@
         <v>28</v>
       </c>
       <c r="D852" s="0" t="s">
-        <v>3802</v>
+        <v>3804</v>
       </c>
       <c r="E852" s="0" t="s">
         <v>66</v>
@@ -56700,10 +56736,10 @@
         <v>32</v>
       </c>
       <c r="H852" s="0" t="s">
-        <v>3803</v>
+        <v>3805</v>
       </c>
       <c r="I852" s="0" t="s">
-        <v>3804</v>
+        <v>3806</v>
       </c>
       <c r="J852" s="0" t="s">
         <v>454</v>
@@ -56718,7 +56754,7 @@
         <v>38</v>
       </c>
       <c r="P852" s="0" t="s">
-        <v>3801</v>
+        <v>3803</v>
       </c>
       <c r="R852" s="0" t="s">
         <v>1502</v>
@@ -56735,7 +56771,7 @@
         <v>128</v>
       </c>
       <c r="D853" s="0" t="s">
-        <v>3805</v>
+        <v>3807</v>
       </c>
       <c r="E853" s="0" t="s">
         <v>1324</v>
@@ -56747,10 +56783,10 @@
         <v>131</v>
       </c>
       <c r="H853" s="0" t="s">
-        <v>3806</v>
+        <v>3808</v>
       </c>
       <c r="I853" s="0" t="s">
-        <v>3807</v>
+        <v>3809</v>
       </c>
       <c r="J853" s="0" t="s">
         <v>924</v>
@@ -56768,10 +56804,10 @@
         <v>2912</v>
       </c>
       <c r="S853" s="0" t="s">
-        <v>3808</v>
+        <v>3810</v>
       </c>
       <c r="T853" s="0" t="s">
-        <v>3809</v>
+        <v>3811</v>
       </c>
     </row>
     <row r="854">
@@ -56785,7 +56821,7 @@
         <v>128</v>
       </c>
       <c r="D854" s="0" t="s">
-        <v>3808</v>
+        <v>3810</v>
       </c>
       <c r="E854" s="0" t="s">
         <v>1342</v>
@@ -56797,10 +56833,10 @@
         <v>131</v>
       </c>
       <c r="H854" s="0" t="s">
-        <v>3810</v>
+        <v>3812</v>
       </c>
       <c r="I854" s="0" t="s">
-        <v>3811</v>
+        <v>3813</v>
       </c>
       <c r="J854" s="0" t="s">
         <v>108</v>
@@ -56829,7 +56865,7 @@
         <v>128</v>
       </c>
       <c r="D855" s="0" t="s">
-        <v>3809</v>
+        <v>3811</v>
       </c>
       <c r="E855" s="0" t="s">
         <v>1342</v>
@@ -56841,10 +56877,10 @@
         <v>131</v>
       </c>
       <c r="H855" s="0" t="s">
-        <v>3812</v>
+        <v>3814</v>
       </c>
       <c r="I855" s="0" t="s">
-        <v>3813</v>
+        <v>3815</v>
       </c>
       <c r="J855" s="0" t="s">
         <v>108</v>
@@ -56870,7 +56906,7 @@
         <v>128</v>
       </c>
       <c r="D856" s="0" t="s">
-        <v>3814</v>
+        <v>3816</v>
       </c>
       <c r="E856" s="0" t="s">
         <v>1466</v>
@@ -56882,10 +56918,10 @@
         <v>131</v>
       </c>
       <c r="H856" s="0" t="s">
-        <v>3815</v>
+        <v>3817</v>
       </c>
       <c r="I856" s="0" t="s">
-        <v>3816</v>
+        <v>3818</v>
       </c>
       <c r="J856" s="0" t="s">
         <v>403</v>
@@ -56894,19 +56930,19 @@
         <v>201</v>
       </c>
       <c r="L856" s="0" t="s">
-        <v>3817</v>
+        <v>3819</v>
       </c>
       <c r="O856" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P856" s="0" t="s">
-        <v>3818</v>
+        <v>3820</v>
       </c>
       <c r="R856" s="0" t="s">
-        <v>3819</v>
+        <v>3821</v>
       </c>
       <c r="S856" s="0" t="s">
-        <v>3820</v>
+        <v>3822</v>
       </c>
     </row>
     <row r="857">
@@ -56920,7 +56956,7 @@
         <v>128</v>
       </c>
       <c r="D857" s="0" t="s">
-        <v>3820</v>
+        <v>3822</v>
       </c>
       <c r="E857" s="0" t="s">
         <v>1342</v>
@@ -56932,10 +56968,10 @@
         <v>131</v>
       </c>
       <c r="H857" s="0" t="s">
-        <v>3821</v>
+        <v>3823</v>
       </c>
       <c r="I857" s="0" t="s">
-        <v>3822</v>
+        <v>3824</v>
       </c>
       <c r="J857" s="0" t="s">
         <v>454</v>
@@ -56944,16 +56980,16 @@
         <v>50</v>
       </c>
       <c r="L857" s="0" t="s">
-        <v>3817</v>
+        <v>3819</v>
       </c>
       <c r="O857" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P857" s="0" t="s">
-        <v>3818</v>
+        <v>3820</v>
       </c>
       <c r="R857" s="0" t="s">
-        <v>3819</v>
+        <v>3821</v>
       </c>
     </row>
     <row r="858">
@@ -56967,7 +57003,7 @@
         <v>28</v>
       </c>
       <c r="D858" s="0" t="s">
-        <v>3823</v>
+        <v>3825</v>
       </c>
       <c r="E858" s="0" t="s">
         <v>66</v>
@@ -56979,10 +57015,10 @@
         <v>32</v>
       </c>
       <c r="H858" s="0" t="s">
-        <v>3824</v>
+        <v>3826</v>
       </c>
       <c r="I858" s="0" t="s">
-        <v>3825</v>
+        <v>3827</v>
       </c>
       <c r="J858" s="0" t="s">
         <v>528</v>
@@ -56991,7 +57027,7 @@
         <v>161</v>
       </c>
       <c r="L858" s="0" t="s">
-        <v>3826</v>
+        <v>3828</v>
       </c>
       <c r="O858" s="0" t="s">
         <v>51</v>
@@ -57000,7 +57036,7 @@
         <v>540</v>
       </c>
       <c r="R858" s="0" t="s">
-        <v>3827</v>
+        <v>3829</v>
       </c>
     </row>
     <row r="859">
@@ -57014,7 +57050,7 @@
         <v>28</v>
       </c>
       <c r="D859" s="0" t="s">
-        <v>3828</v>
+        <v>3830</v>
       </c>
       <c r="E859" s="0" t="s">
         <v>66</v>
@@ -57026,10 +57062,10 @@
         <v>32</v>
       </c>
       <c r="H859" s="0" t="s">
-        <v>3829</v>
+        <v>3831</v>
       </c>
       <c r="I859" s="0" t="s">
-        <v>3830</v>
+        <v>3832</v>
       </c>
       <c r="J859" s="0" t="s">
         <v>528</v>
@@ -57038,7 +57074,7 @@
         <v>161</v>
       </c>
       <c r="L859" s="0" t="s">
-        <v>3826</v>
+        <v>3828</v>
       </c>
       <c r="O859" s="0" t="s">
         <v>51</v>
@@ -57047,7 +57083,7 @@
         <v>540</v>
       </c>
       <c r="R859" s="0" t="s">
-        <v>3827</v>
+        <v>3829</v>
       </c>
     </row>
     <row r="860">
@@ -57061,7 +57097,7 @@
         <v>28</v>
       </c>
       <c r="D860" s="0" t="s">
-        <v>3831</v>
+        <v>3833</v>
       </c>
       <c r="E860" s="0" t="s">
         <v>76</v>
@@ -57073,10 +57109,10 @@
         <v>32</v>
       </c>
       <c r="H860" s="0" t="s">
-        <v>3832</v>
+        <v>3834</v>
       </c>
       <c r="I860" s="0" t="s">
-        <v>3833</v>
+        <v>3835</v>
       </c>
       <c r="J860" s="0" t="s">
         <v>97</v>
@@ -57097,10 +57133,10 @@
         <v>53</v>
       </c>
       <c r="S860" s="0" t="s">
-        <v>3834</v>
+        <v>3836</v>
       </c>
       <c r="T860" s="0" t="s">
-        <v>3835</v>
+        <v>3837</v>
       </c>
     </row>
     <row r="861">
@@ -57114,7 +57150,7 @@
         <v>28</v>
       </c>
       <c r="D861" s="0" t="s">
-        <v>3835</v>
+        <v>3837</v>
       </c>
       <c r="E861" s="0" t="s">
         <v>66</v>
@@ -57126,10 +57162,10 @@
         <v>32</v>
       </c>
       <c r="H861" s="0" t="s">
-        <v>3836</v>
+        <v>3838</v>
       </c>
       <c r="I861" s="0" t="s">
-        <v>3837</v>
+        <v>3839</v>
       </c>
       <c r="J861" s="0" t="s">
         <v>35</v>
@@ -57161,7 +57197,7 @@
         <v>28</v>
       </c>
       <c r="D862" s="0" t="s">
-        <v>3834</v>
+        <v>3836</v>
       </c>
       <c r="E862" s="0" t="s">
         <v>66</v>
@@ -57173,10 +57209,10 @@
         <v>32</v>
       </c>
       <c r="H862" s="0" t="s">
-        <v>3838</v>
+        <v>3840</v>
       </c>
       <c r="I862" s="0" t="s">
-        <v>3839</v>
+        <v>3841</v>
       </c>
       <c r="J862" s="0" t="s">
         <v>35</v>
@@ -57208,7 +57244,7 @@
         <v>28</v>
       </c>
       <c r="D863" s="0" t="s">
-        <v>3840</v>
+        <v>3842</v>
       </c>
       <c r="E863" s="0" t="s">
         <v>76</v>
@@ -57220,10 +57256,10 @@
         <v>32</v>
       </c>
       <c r="H863" s="0" t="s">
-        <v>3841</v>
+        <v>3843</v>
       </c>
       <c r="I863" s="0" t="s">
-        <v>3842</v>
+        <v>3844</v>
       </c>
       <c r="J863" s="0" t="s">
         <v>665</v>
@@ -57238,13 +57274,13 @@
         <v>38</v>
       </c>
       <c r="P863" s="0" t="s">
-        <v>3843</v>
+        <v>3845</v>
       </c>
       <c r="R863" s="0" t="s">
-        <v>3844</v>
+        <v>3846</v>
       </c>
       <c r="S863" s="0" t="s">
-        <v>3845</v>
+        <v>3847</v>
       </c>
     </row>
     <row r="864">
@@ -57258,22 +57294,22 @@
         <v>28</v>
       </c>
       <c r="D864" s="0" t="s">
-        <v>3845</v>
+        <v>3847</v>
       </c>
       <c r="E864" s="0" t="s">
         <v>45</v>
       </c>
       <c r="F864" s="0" t="s">
-        <v>3846</v>
+        <v>3848</v>
       </c>
       <c r="G864" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H864" s="0" t="s">
-        <v>3847</v>
+        <v>3849</v>
       </c>
       <c r="I864" s="0" t="s">
-        <v>3848</v>
+        <v>3850</v>
       </c>
       <c r="J864" s="0" t="s">
         <v>454</v>
@@ -57282,13 +57318,13 @@
         <v>50</v>
       </c>
       <c r="L864" s="0" t="s">
-        <v>3849</v>
+        <v>3851</v>
       </c>
       <c r="O864" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P864" s="0" t="s">
-        <v>3843</v>
+        <v>3845</v>
       </c>
     </row>
     <row r="865">
@@ -57314,10 +57350,10 @@
         <v>32</v>
       </c>
       <c r="H865" s="0" t="s">
-        <v>3850</v>
+        <v>3852</v>
       </c>
       <c r="I865" s="0" t="s">
-        <v>3851</v>
+        <v>3853</v>
       </c>
       <c r="J865" s="0" t="s">
         <v>746</v>
@@ -57346,7 +57382,7 @@
         <v>28</v>
       </c>
       <c r="D866" s="0" t="s">
-        <v>3852</v>
+        <v>3854</v>
       </c>
       <c r="E866" s="0" t="s">
         <v>60</v>
@@ -57358,10 +57394,10 @@
         <v>32</v>
       </c>
       <c r="H866" s="0" t="s">
-        <v>3853</v>
+        <v>3855</v>
       </c>
       <c r="I866" s="0" t="s">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="J866" s="0" t="s">
         <v>1701</v>
@@ -57376,13 +57412,13 @@
         <v>38</v>
       </c>
       <c r="P866" s="0" t="s">
-        <v>3855</v>
+        <v>3857</v>
       </c>
       <c r="R866" s="0" t="s">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="S866" s="0" t="s">
-        <v>3857</v>
+        <v>3859</v>
       </c>
     </row>
     <row r="867">
@@ -57396,22 +57432,22 @@
         <v>28</v>
       </c>
       <c r="D867" s="0" t="s">
-        <v>3857</v>
+        <v>3859</v>
       </c>
       <c r="E867" s="0" t="s">
         <v>357</v>
       </c>
       <c r="F867" s="0" t="s">
-        <v>3858</v>
+        <v>3860</v>
       </c>
       <c r="G867" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H867" s="0" t="s">
-        <v>3859</v>
+        <v>3861</v>
       </c>
       <c r="I867" s="0" t="s">
-        <v>3860</v>
+        <v>3862</v>
       </c>
       <c r="J867" s="0" t="s">
         <v>423</v>
@@ -57426,7 +57462,7 @@
         <v>38</v>
       </c>
       <c r="P867" s="0" t="s">
-        <v>3861</v>
+        <v>3863</v>
       </c>
     </row>
     <row r="868">
@@ -57440,7 +57476,7 @@
         <v>28</v>
       </c>
       <c r="D868" s="0" t="s">
-        <v>3862</v>
+        <v>3864</v>
       </c>
       <c r="E868" s="0" t="s">
         <v>196</v>
@@ -57452,10 +57488,10 @@
         <v>32</v>
       </c>
       <c r="H868" s="0" t="s">
-        <v>3863</v>
+        <v>3865</v>
       </c>
       <c r="I868" s="0" t="s">
-        <v>3864</v>
+        <v>3866</v>
       </c>
       <c r="J868" s="0" t="s">
         <v>535</v>
@@ -57464,22 +57500,22 @@
         <v>36</v>
       </c>
       <c r="L868" s="0" t="s">
-        <v>3865</v>
+        <v>3867</v>
       </c>
       <c r="O868" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P868" s="0" t="s">
-        <v>3866</v>
+        <v>3868</v>
       </c>
       <c r="R868" s="0" t="s">
-        <v>3862</v>
+        <v>3864</v>
       </c>
       <c r="S868" s="0" t="s">
-        <v>3867</v>
+        <v>3869</v>
       </c>
       <c r="T868" s="0" t="s">
-        <v>3868</v>
+        <v>3870</v>
       </c>
     </row>
     <row r="869">
@@ -57493,7 +57529,7 @@
         <v>28</v>
       </c>
       <c r="D869" s="0" t="s">
-        <v>3867</v>
+        <v>3869</v>
       </c>
       <c r="E869" s="0" t="s">
         <v>104</v>
@@ -57505,10 +57541,10 @@
         <v>32</v>
       </c>
       <c r="H869" s="0" t="s">
-        <v>3869</v>
+        <v>3871</v>
       </c>
       <c r="I869" s="0" t="s">
-        <v>3870</v>
+        <v>3872</v>
       </c>
       <c r="J869" s="0" t="s">
         <v>49</v>
@@ -57523,10 +57559,10 @@
         <v>38</v>
       </c>
       <c r="P869" s="0" t="s">
-        <v>3866</v>
+        <v>3868</v>
       </c>
       <c r="R869" s="0" t="s">
-        <v>3871</v>
+        <v>3873</v>
       </c>
     </row>
     <row r="870">
@@ -57540,7 +57576,7 @@
         <v>28</v>
       </c>
       <c r="D870" s="0" t="s">
-        <v>3868</v>
+        <v>3870</v>
       </c>
       <c r="E870" s="0" t="s">
         <v>104</v>
@@ -57552,10 +57588,10 @@
         <v>32</v>
       </c>
       <c r="H870" s="0" t="s">
-        <v>3872</v>
+        <v>3874</v>
       </c>
       <c r="I870" s="0" t="s">
-        <v>3873</v>
+        <v>3875</v>
       </c>
       <c r="J870" s="0" t="s">
         <v>49</v>
@@ -57570,10 +57606,10 @@
         <v>38</v>
       </c>
       <c r="P870" s="0" t="s">
-        <v>3866</v>
+        <v>3868</v>
       </c>
       <c r="R870" s="0" t="s">
-        <v>3871</v>
+        <v>3873</v>
       </c>
     </row>
     <row r="871">
@@ -57587,22 +57623,22 @@
         <v>128</v>
       </c>
       <c r="D871" s="0" t="s">
-        <v>3874</v>
+        <v>3876</v>
       </c>
       <c r="E871" s="0" t="s">
-        <v>3875</v>
+        <v>3877</v>
       </c>
       <c r="F871" s="0" t="s">
-        <v>3875</v>
+        <v>3877</v>
       </c>
       <c r="G871" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H871" s="0" t="s">
-        <v>3876</v>
+        <v>3878</v>
       </c>
       <c r="I871" s="0" t="s">
-        <v>3877</v>
+        <v>3879</v>
       </c>
       <c r="J871" s="0" t="s">
         <v>160</v>
@@ -57617,7 +57653,7 @@
         <v>38</v>
       </c>
       <c r="R871" s="0" t="s">
-        <v>3878</v>
+        <v>3880</v>
       </c>
       <c r="S871" s="0" t="s">
         <v>2902</v>
@@ -57637,7 +57673,7 @@
         <v>28</v>
       </c>
       <c r="D872" s="0" t="s">
-        <v>3879</v>
+        <v>3881</v>
       </c>
       <c r="E872" s="0" t="s">
         <v>30</v>
@@ -57649,10 +57685,10 @@
         <v>32</v>
       </c>
       <c r="H872" s="0" t="s">
-        <v>3880</v>
+        <v>3882</v>
       </c>
       <c r="I872" s="0" t="s">
-        <v>3881</v>
+        <v>3883</v>
       </c>
       <c r="J872" s="0" t="s">
         <v>108</v>
@@ -57699,10 +57735,10 @@
         <v>32</v>
       </c>
       <c r="H873" s="0" t="s">
-        <v>3882</v>
+        <v>3884</v>
       </c>
       <c r="I873" s="0" t="s">
-        <v>3883</v>
+        <v>3885</v>
       </c>
       <c r="J873" s="0" t="s">
         <v>142</v>
@@ -57717,7 +57753,7 @@
         <v>38</v>
       </c>
       <c r="P873" s="0" t="s">
-        <v>3884</v>
+        <v>3886</v>
       </c>
       <c r="R873" s="0" t="s">
         <v>3298</v>
@@ -57746,10 +57782,10 @@
         <v>32</v>
       </c>
       <c r="H874" s="0" t="s">
-        <v>3885</v>
+        <v>3887</v>
       </c>
       <c r="I874" s="0" t="s">
-        <v>3886</v>
+        <v>3888</v>
       </c>
       <c r="J874" s="0" t="s">
         <v>142</v>
@@ -57764,7 +57800,7 @@
         <v>38</v>
       </c>
       <c r="P874" s="0" t="s">
-        <v>3884</v>
+        <v>3886</v>
       </c>
       <c r="R874" s="0" t="s">
         <v>3298</v>
@@ -57781,7 +57817,7 @@
         <v>128</v>
       </c>
       <c r="D875" s="0" t="s">
-        <v>3887</v>
+        <v>3889</v>
       </c>
       <c r="E875" s="0" t="s">
         <v>1293</v>
@@ -57793,10 +57829,10 @@
         <v>131</v>
       </c>
       <c r="H875" s="0" t="s">
-        <v>3888</v>
+        <v>3890</v>
       </c>
       <c r="I875" s="0" t="s">
-        <v>3889</v>
+        <v>3891</v>
       </c>
       <c r="J875" s="0" t="s">
         <v>341</v>
@@ -57811,10 +57847,10 @@
         <v>51</v>
       </c>
       <c r="R875" s="0" t="s">
-        <v>3890</v>
+        <v>3892</v>
       </c>
       <c r="S875" s="0" t="s">
-        <v>3891</v>
+        <v>3893</v>
       </c>
     </row>
     <row r="876">
@@ -57828,22 +57864,22 @@
         <v>128</v>
       </c>
       <c r="D876" s="0" t="s">
-        <v>3892</v>
+        <v>3894</v>
       </c>
       <c r="E876" s="0" t="s">
-        <v>3893</v>
+        <v>3895</v>
       </c>
       <c r="F876" s="0" t="s">
-        <v>3893</v>
+        <v>3895</v>
       </c>
       <c r="G876" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H876" s="0" t="s">
-        <v>3894</v>
+        <v>3896</v>
       </c>
       <c r="I876" s="0" t="s">
-        <v>3895</v>
+        <v>3897</v>
       </c>
       <c r="J876" s="0" t="s">
         <v>535</v>
@@ -57852,13 +57888,13 @@
         <v>36</v>
       </c>
       <c r="L876" s="0" t="s">
-        <v>3896</v>
+        <v>3898</v>
       </c>
       <c r="O876" s="0" t="s">
         <v>51</v>
       </c>
       <c r="R876" s="0" t="s">
-        <v>3890</v>
+        <v>3892</v>
       </c>
     </row>
     <row r="877">
@@ -57872,22 +57908,22 @@
         <v>128</v>
       </c>
       <c r="D877" s="0" t="s">
-        <v>3897</v>
+        <v>3899</v>
       </c>
       <c r="E877" s="0" t="s">
-        <v>3898</v>
+        <v>3900</v>
       </c>
       <c r="F877" s="0" t="s">
-        <v>3898</v>
+        <v>3900</v>
       </c>
       <c r="G877" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H877" s="0" t="s">
-        <v>3899</v>
+        <v>3901</v>
       </c>
       <c r="I877" s="0" t="s">
-        <v>3900</v>
+        <v>3902</v>
       </c>
       <c r="J877" s="0" t="s">
         <v>924</v>
@@ -57902,7 +57938,7 @@
         <v>51</v>
       </c>
       <c r="R877" s="0" t="s">
-        <v>3901</v>
+        <v>3903</v>
       </c>
     </row>
     <row r="878">
@@ -57916,7 +57952,7 @@
         <v>91</v>
       </c>
       <c r="D878" s="0" t="s">
-        <v>3902</v>
+        <v>3904</v>
       </c>
       <c r="E878" s="0" t="s">
         <v>196</v>
@@ -57928,10 +57964,10 @@
         <v>94</v>
       </c>
       <c r="H878" s="0" t="s">
-        <v>3903</v>
+        <v>3905</v>
       </c>
       <c r="I878" s="0" t="s">
-        <v>3904</v>
+        <v>3906</v>
       </c>
       <c r="J878" s="0" t="s">
         <v>80</v>
@@ -57946,10 +57982,10 @@
         <v>51</v>
       </c>
       <c r="P878" s="0" t="s">
-        <v>3905</v>
+        <v>3907</v>
       </c>
       <c r="R878" s="0" t="s">
-        <v>3906</v>
+        <v>3908</v>
       </c>
     </row>
     <row r="879">
@@ -57963,22 +57999,22 @@
         <v>128</v>
       </c>
       <c r="D879" s="0" t="s">
-        <v>3907</v>
+        <v>3909</v>
       </c>
       <c r="E879" s="0" t="s">
-        <v>3908</v>
+        <v>3910</v>
       </c>
       <c r="F879" s="0" t="s">
-        <v>3908</v>
+        <v>3910</v>
       </c>
       <c r="G879" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H879" s="0" t="s">
-        <v>3909</v>
+        <v>3911</v>
       </c>
       <c r="I879" s="0" t="s">
-        <v>3910</v>
+        <v>3912</v>
       </c>
       <c r="J879" s="0" t="s">
         <v>35</v>
@@ -57993,10 +58029,10 @@
         <v>38</v>
       </c>
       <c r="R879" s="0" t="s">
-        <v>3911</v>
+        <v>3913</v>
       </c>
       <c r="S879" s="0" t="s">
-        <v>3912</v>
+        <v>3914</v>
       </c>
     </row>
     <row r="880">
@@ -58010,7 +58046,7 @@
         <v>128</v>
       </c>
       <c r="D880" s="0" t="s">
-        <v>3912</v>
+        <v>3914</v>
       </c>
       <c r="E880" s="0" t="s">
         <v>1342</v>
@@ -58022,10 +58058,10 @@
         <v>131</v>
       </c>
       <c r="H880" s="0" t="s">
-        <v>3913</v>
+        <v>3915</v>
       </c>
       <c r="I880" s="0" t="s">
-        <v>3914</v>
+        <v>3916</v>
       </c>
       <c r="J880" s="0" t="s">
         <v>108</v>
@@ -58040,7 +58076,7 @@
         <v>38</v>
       </c>
       <c r="R880" s="0" t="s">
-        <v>3911</v>
+        <v>3913</v>
       </c>
     </row>
     <row r="881">
@@ -58054,7 +58090,7 @@
         <v>128</v>
       </c>
       <c r="D881" s="0" t="s">
-        <v>3915</v>
+        <v>3917</v>
       </c>
       <c r="E881" s="0" t="s">
         <v>1293</v>
@@ -58066,10 +58102,10 @@
         <v>131</v>
       </c>
       <c r="H881" s="0" t="s">
-        <v>3916</v>
+        <v>3918</v>
       </c>
       <c r="I881" s="0" t="s">
-        <v>3917</v>
+        <v>3919</v>
       </c>
       <c r="J881" s="0" t="s">
         <v>913</v>
@@ -58078,19 +58114,19 @@
         <v>201</v>
       </c>
       <c r="L881" s="0" t="s">
-        <v>3918</v>
+        <v>3920</v>
       </c>
       <c r="O881" s="0" t="s">
         <v>51</v>
       </c>
       <c r="R881" s="0" t="s">
-        <v>3919</v>
+        <v>3921</v>
       </c>
       <c r="S881" s="0" t="s">
-        <v>3920</v>
+        <v>3922</v>
       </c>
       <c r="T881" s="0" t="s">
-        <v>3921</v>
+        <v>3923</v>
       </c>
     </row>
     <row r="882">
@@ -58104,7 +58140,7 @@
         <v>128</v>
       </c>
       <c r="D882" s="0" t="s">
-        <v>3920</v>
+        <v>3922</v>
       </c>
       <c r="E882" s="0" t="s">
         <v>1298</v>
@@ -58116,10 +58152,10 @@
         <v>131</v>
       </c>
       <c r="H882" s="0" t="s">
-        <v>3922</v>
+        <v>3924</v>
       </c>
       <c r="I882" s="0" t="s">
-        <v>3923</v>
+        <v>3925</v>
       </c>
       <c r="J882" s="0" t="s">
         <v>396</v>
@@ -58128,13 +58164,13 @@
         <v>71</v>
       </c>
       <c r="L882" s="0" t="s">
-        <v>3918</v>
+        <v>3920</v>
       </c>
       <c r="O882" s="0" t="s">
         <v>51</v>
       </c>
       <c r="R882" s="0" t="s">
-        <v>3919</v>
+        <v>3921</v>
       </c>
     </row>
     <row r="883">
@@ -58148,7 +58184,7 @@
         <v>128</v>
       </c>
       <c r="D883" s="0" t="s">
-        <v>3921</v>
+        <v>3923</v>
       </c>
       <c r="E883" s="0" t="s">
         <v>1302</v>
@@ -58160,10 +58196,10 @@
         <v>131</v>
       </c>
       <c r="H883" s="0" t="s">
-        <v>3924</v>
+        <v>3926</v>
       </c>
       <c r="I883" s="0" t="s">
-        <v>3925</v>
+        <v>3927</v>
       </c>
       <c r="J883" s="0" t="s">
         <v>396</v>
@@ -58172,13 +58208,13 @@
         <v>71</v>
       </c>
       <c r="L883" s="0" t="s">
-        <v>3918</v>
+        <v>3920</v>
       </c>
       <c r="O883" s="0" t="s">
         <v>51</v>
       </c>
       <c r="R883" s="0" t="s">
-        <v>3919</v>
+        <v>3921</v>
       </c>
     </row>
     <row r="884">
@@ -58192,7 +58228,7 @@
         <v>128</v>
       </c>
       <c r="D884" s="0" t="s">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="E884" s="0" t="s">
         <v>1175</v>
@@ -58204,10 +58240,10 @@
         <v>131</v>
       </c>
       <c r="H884" s="0" t="s">
-        <v>3927</v>
+        <v>3929</v>
       </c>
       <c r="I884" s="0" t="s">
-        <v>3928</v>
+        <v>3930</v>
       </c>
       <c r="J884" s="0" t="s">
         <v>200</v>
@@ -58222,7 +58258,7 @@
         <v>51</v>
       </c>
       <c r="R884" s="0" t="s">
-        <v>3929</v>
+        <v>3931</v>
       </c>
     </row>
     <row r="885">
@@ -58236,22 +58272,22 @@
         <v>28</v>
       </c>
       <c r="D885" s="0" t="s">
-        <v>3930</v>
+        <v>3932</v>
       </c>
       <c r="E885" s="0" t="s">
         <v>1850</v>
       </c>
       <c r="F885" s="0" t="s">
-        <v>3931</v>
+        <v>3933</v>
       </c>
       <c r="G885" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H885" s="0" t="s">
-        <v>3932</v>
+        <v>3934</v>
       </c>
       <c r="I885" s="0" t="s">
-        <v>3933</v>
+        <v>3935</v>
       </c>
       <c r="J885" s="0" t="s">
         <v>280</v>
@@ -58266,7 +58302,7 @@
         <v>38</v>
       </c>
       <c r="P885" s="0" t="s">
-        <v>3884</v>
+        <v>3886</v>
       </c>
       <c r="R885" s="0" t="s">
         <v>3298</v>
@@ -58289,7 +58325,7 @@
         <v>128</v>
       </c>
       <c r="D886" s="0" t="s">
-        <v>3934</v>
+        <v>3936</v>
       </c>
       <c r="E886" s="0" t="s">
         <v>1166</v>
@@ -58319,10 +58355,10 @@
         <v>38</v>
       </c>
       <c r="R886" s="0" t="s">
-        <v>3935</v>
+        <v>3937</v>
       </c>
       <c r="S886" s="0" t="s">
-        <v>3936</v>
+        <v>3938</v>
       </c>
     </row>
     <row r="887">
@@ -58336,22 +58372,22 @@
         <v>128</v>
       </c>
       <c r="D887" s="0" t="s">
-        <v>3936</v>
+        <v>3938</v>
       </c>
       <c r="E887" s="0" t="s">
-        <v>3937</v>
+        <v>3939</v>
       </c>
       <c r="F887" s="0" t="s">
-        <v>3937</v>
+        <v>3939</v>
       </c>
       <c r="G887" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H887" s="0" t="s">
-        <v>3938</v>
+        <v>3940</v>
       </c>
       <c r="I887" s="0" t="s">
-        <v>3939</v>
+        <v>3941</v>
       </c>
       <c r="J887" s="0" t="s">
         <v>300</v>
@@ -58366,7 +58402,7 @@
         <v>38</v>
       </c>
       <c r="R887" s="0" t="s">
-        <v>3935</v>
+        <v>3937</v>
       </c>
     </row>
     <row r="888">
@@ -58380,22 +58416,22 @@
         <v>91</v>
       </c>
       <c r="D888" s="0" t="s">
-        <v>3940</v>
+        <v>3942</v>
       </c>
       <c r="E888" s="0" t="s">
         <v>256</v>
       </c>
       <c r="F888" s="0" t="s">
-        <v>3941</v>
+        <v>3943</v>
       </c>
       <c r="G888" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H888" s="0" t="s">
-        <v>3942</v>
+        <v>3944</v>
       </c>
       <c r="I888" s="0" t="s">
-        <v>3943</v>
+        <v>3945</v>
       </c>
       <c r="J888" s="0" t="s">
         <v>97</v>
@@ -58413,10 +58449,10 @@
         <v>334</v>
       </c>
       <c r="R888" s="0" t="s">
-        <v>3944</v>
+        <v>3946</v>
       </c>
       <c r="S888" s="0" t="s">
-        <v>3945</v>
+        <v>3947</v>
       </c>
     </row>
     <row r="889">
@@ -58430,7 +58466,7 @@
         <v>91</v>
       </c>
       <c r="D889" s="0" t="s">
-        <v>3946</v>
+        <v>3948</v>
       </c>
       <c r="E889" s="0" t="s">
         <v>60</v>
@@ -58442,10 +58478,10 @@
         <v>94</v>
       </c>
       <c r="H889" s="0" t="s">
-        <v>3947</v>
+        <v>3949</v>
       </c>
       <c r="I889" s="0" t="s">
-        <v>3948</v>
+        <v>3950</v>
       </c>
       <c r="J889" s="0" t="s">
         <v>288</v>
@@ -58460,13 +58496,13 @@
         <v>38</v>
       </c>
       <c r="P889" s="0" t="s">
-        <v>3949</v>
+        <v>3951</v>
       </c>
       <c r="R889" s="0" t="s">
-        <v>3950</v>
+        <v>3952</v>
       </c>
       <c r="S889" s="0" t="s">
-        <v>3951</v>
+        <v>3953</v>
       </c>
     </row>
     <row r="890">
@@ -58480,22 +58516,22 @@
         <v>91</v>
       </c>
       <c r="D890" s="0" t="s">
-        <v>3952</v>
+        <v>3954</v>
       </c>
       <c r="E890" s="0" t="s">
         <v>76</v>
       </c>
       <c r="F890" s="0" t="s">
-        <v>3953</v>
+        <v>3955</v>
       </c>
       <c r="G890" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H890" s="0" t="s">
-        <v>3954</v>
+        <v>3956</v>
       </c>
       <c r="I890" s="0" t="s">
-        <v>3955</v>
+        <v>3957</v>
       </c>
       <c r="J890" s="0" t="s">
         <v>1034</v>
@@ -58510,13 +58546,13 @@
         <v>38</v>
       </c>
       <c r="P890" s="0" t="s">
-        <v>3956</v>
+        <v>3958</v>
       </c>
       <c r="R890" s="0" t="s">
-        <v>3957</v>
+        <v>3959</v>
       </c>
       <c r="S890" s="0" t="s">
-        <v>3958</v>
+        <v>3960</v>
       </c>
     </row>
     <row r="891">
@@ -58530,7 +58566,7 @@
         <v>91</v>
       </c>
       <c r="D891" s="0" t="s">
-        <v>3959</v>
+        <v>3961</v>
       </c>
       <c r="E891" s="0" t="s">
         <v>214</v>
@@ -58542,10 +58578,10 @@
         <v>94</v>
       </c>
       <c r="H891" s="0" t="s">
-        <v>3960</v>
+        <v>3962</v>
       </c>
       <c r="I891" s="0" t="s">
-        <v>3961</v>
+        <v>3963</v>
       </c>
       <c r="J891" s="0" t="s">
         <v>280</v>
@@ -58560,10 +58596,10 @@
         <v>51</v>
       </c>
       <c r="P891" s="0" t="s">
-        <v>3962</v>
+        <v>3964</v>
       </c>
       <c r="R891" s="0" t="s">
-        <v>3963</v>
+        <v>3965</v>
       </c>
     </row>
     <row r="892">
@@ -58577,7 +58613,7 @@
         <v>91</v>
       </c>
       <c r="D892" s="0" t="s">
-        <v>3964</v>
+        <v>3966</v>
       </c>
       <c r="E892" s="0" t="s">
         <v>76</v>
@@ -58589,10 +58625,10 @@
         <v>94</v>
       </c>
       <c r="H892" s="0" t="s">
-        <v>3965</v>
+        <v>3967</v>
       </c>
       <c r="I892" s="0" t="s">
-        <v>3966</v>
+        <v>3968</v>
       </c>
       <c r="J892" s="0" t="s">
         <v>352</v>
@@ -58607,13 +58643,13 @@
         <v>38</v>
       </c>
       <c r="P892" s="0" t="s">
-        <v>3967</v>
+        <v>3969</v>
       </c>
       <c r="R892" s="0" t="s">
-        <v>3968</v>
+        <v>3970</v>
       </c>
       <c r="S892" s="0" t="s">
-        <v>3969</v>
+        <v>3971</v>
       </c>
     </row>
     <row r="893">
@@ -58627,22 +58663,22 @@
         <v>91</v>
       </c>
       <c r="D893" s="0" t="s">
-        <v>3970</v>
+        <v>3972</v>
       </c>
       <c r="E893" s="0" t="s">
         <v>196</v>
       </c>
       <c r="F893" s="0" t="s">
-        <v>3971</v>
+        <v>3973</v>
       </c>
       <c r="G893" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H893" s="0" t="s">
-        <v>3972</v>
+        <v>3974</v>
       </c>
       <c r="I893" s="0" t="s">
-        <v>3973</v>
+        <v>3975</v>
       </c>
       <c r="J893" s="0" t="s">
         <v>746</v>
@@ -58651,7 +58687,7 @@
         <v>201</v>
       </c>
       <c r="L893" s="0" t="s">
-        <v>3974</v>
+        <v>3976</v>
       </c>
       <c r="O893" s="0" t="s">
         <v>38</v>
@@ -58677,7 +58713,7 @@
         <v>91</v>
       </c>
       <c r="D894" s="0" t="s">
-        <v>3975</v>
+        <v>3977</v>
       </c>
       <c r="E894" s="0" t="s">
         <v>76</v>
@@ -58689,10 +58725,10 @@
         <v>94</v>
       </c>
       <c r="H894" s="0" t="s">
-        <v>3976</v>
+        <v>3978</v>
       </c>
       <c r="I894" s="0" t="s">
-        <v>3977</v>
+        <v>3979</v>
       </c>
       <c r="J894" s="0" t="s">
         <v>403</v>
@@ -58701,19 +58737,19 @@
         <v>201</v>
       </c>
       <c r="L894" s="0" t="s">
-        <v>3978</v>
+        <v>3980</v>
       </c>
       <c r="O894" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P894" s="0" t="s">
-        <v>3979</v>
+        <v>3981</v>
       </c>
       <c r="R894" s="0" t="s">
-        <v>3980</v>
+        <v>3982</v>
       </c>
       <c r="S894" s="0" t="s">
-        <v>3981</v>
+        <v>3983</v>
       </c>
     </row>
     <row r="895">
@@ -58727,22 +58763,22 @@
         <v>91</v>
       </c>
       <c r="D895" s="0" t="s">
-        <v>3982</v>
+        <v>3984</v>
       </c>
       <c r="E895" s="0" t="s">
         <v>196</v>
       </c>
       <c r="F895" s="0" t="s">
-        <v>3983</v>
+        <v>3985</v>
       </c>
       <c r="G895" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H895" s="0" t="s">
-        <v>3984</v>
+        <v>3986</v>
       </c>
       <c r="I895" s="0" t="s">
-        <v>3985</v>
+        <v>3987</v>
       </c>
       <c r="J895" s="0" t="s">
         <v>243</v>
@@ -58757,10 +58793,10 @@
         <v>38</v>
       </c>
       <c r="P895" s="0" t="s">
-        <v>3986</v>
+        <v>3988</v>
       </c>
       <c r="R895" s="0" t="s">
-        <v>3987</v>
+        <v>3989</v>
       </c>
     </row>
     <row r="896">
@@ -58774,7 +58810,7 @@
         <v>91</v>
       </c>
       <c r="D896" s="0" t="s">
-        <v>3988</v>
+        <v>3990</v>
       </c>
       <c r="E896" s="0" t="s">
         <v>60</v>
@@ -58786,10 +58822,10 @@
         <v>94</v>
       </c>
       <c r="H896" s="0" t="s">
-        <v>3989</v>
+        <v>3991</v>
       </c>
       <c r="I896" s="0" t="s">
-        <v>3990</v>
+        <v>3992</v>
       </c>
       <c r="J896" s="0" t="s">
         <v>300</v>
@@ -58804,13 +58840,13 @@
         <v>38</v>
       </c>
       <c r="P896" s="0" t="s">
-        <v>3991</v>
+        <v>3993</v>
       </c>
       <c r="R896" s="0" t="s">
         <v>3698</v>
       </c>
       <c r="S896" s="0" t="s">
-        <v>3992</v>
+        <v>3994</v>
       </c>
     </row>
     <row r="897">
@@ -58824,7 +58860,7 @@
         <v>91</v>
       </c>
       <c r="D897" s="0" t="s">
-        <v>3945</v>
+        <v>3947</v>
       </c>
       <c r="E897" s="0" t="s">
         <v>759</v>
@@ -58836,10 +58872,10 @@
         <v>94</v>
       </c>
       <c r="H897" s="0" t="s">
-        <v>3993</v>
+        <v>3995</v>
       </c>
       <c r="I897" s="0" t="s">
-        <v>3994</v>
+        <v>3996</v>
       </c>
       <c r="J897" s="0" t="s">
         <v>1034</v>
@@ -58857,7 +58893,7 @@
         <v>334</v>
       </c>
       <c r="R897" s="0" t="s">
-        <v>3944</v>
+        <v>3946</v>
       </c>
     </row>
     <row r="898">
@@ -58877,16 +58913,16 @@
         <v>3099</v>
       </c>
       <c r="F898" s="0" t="s">
-        <v>3995</v>
+        <v>3997</v>
       </c>
       <c r="G898" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H898" s="0" t="s">
-        <v>3996</v>
+        <v>3998</v>
       </c>
       <c r="I898" s="0" t="s">
-        <v>3997</v>
+        <v>3999</v>
       </c>
       <c r="J898" s="0" t="s">
         <v>2905</v>
@@ -58918,7 +58954,7 @@
         <v>91</v>
       </c>
       <c r="D899" s="0" t="s">
-        <v>3951</v>
+        <v>3953</v>
       </c>
       <c r="E899" s="0" t="s">
         <v>759</v>
@@ -58930,10 +58966,10 @@
         <v>94</v>
       </c>
       <c r="H899" s="0" t="s">
-        <v>3998</v>
+        <v>4000</v>
       </c>
       <c r="I899" s="0" t="s">
-        <v>3999</v>
+        <v>4001</v>
       </c>
       <c r="J899" s="0" t="s">
         <v>3089</v>
@@ -58948,10 +58984,10 @@
         <v>38</v>
       </c>
       <c r="P899" s="0" t="s">
-        <v>3949</v>
+        <v>3951</v>
       </c>
       <c r="R899" s="0" t="s">
-        <v>3950</v>
+        <v>3952</v>
       </c>
     </row>
     <row r="900">
@@ -58965,7 +59001,7 @@
         <v>91</v>
       </c>
       <c r="D900" s="0" t="s">
-        <v>3958</v>
+        <v>3960</v>
       </c>
       <c r="E900" s="0" t="s">
         <v>685</v>
@@ -58977,10 +59013,10 @@
         <v>94</v>
       </c>
       <c r="H900" s="0" t="s">
-        <v>4000</v>
+        <v>4002</v>
       </c>
       <c r="I900" s="0" t="s">
-        <v>4001</v>
+        <v>4003</v>
       </c>
       <c r="J900" s="0" t="s">
         <v>568</v>
@@ -58995,10 +59031,10 @@
         <v>38</v>
       </c>
       <c r="P900" s="0" t="s">
-        <v>3956</v>
+        <v>3958</v>
       </c>
       <c r="R900" s="0" t="s">
-        <v>3957</v>
+        <v>3959</v>
       </c>
     </row>
     <row r="901">
@@ -59024,10 +59060,10 @@
         <v>94</v>
       </c>
       <c r="H901" s="0" t="s">
-        <v>4002</v>
+        <v>4004</v>
       </c>
       <c r="I901" s="0" t="s">
-        <v>4003</v>
+        <v>4005</v>
       </c>
       <c r="J901" s="0" t="s">
         <v>108</v>
@@ -59059,22 +59095,22 @@
         <v>91</v>
       </c>
       <c r="D902" s="0" t="s">
-        <v>3969</v>
+        <v>3971</v>
       </c>
       <c r="E902" s="0" t="s">
         <v>685</v>
       </c>
       <c r="F902" s="0" t="s">
-        <v>4004</v>
+        <v>4006</v>
       </c>
       <c r="G902" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H902" s="0" t="s">
-        <v>4005</v>
+        <v>4007</v>
       </c>
       <c r="I902" s="0" t="s">
-        <v>4006</v>
+        <v>4008</v>
       </c>
       <c r="J902" s="0" t="s">
         <v>288</v>
@@ -59089,10 +59125,10 @@
         <v>38</v>
       </c>
       <c r="P902" s="0" t="s">
-        <v>3967</v>
+        <v>3969</v>
       </c>
       <c r="R902" s="0" t="s">
-        <v>3968</v>
+        <v>3970</v>
       </c>
     </row>
     <row r="903">
@@ -59118,10 +59154,10 @@
         <v>94</v>
       </c>
       <c r="H903" s="0" t="s">
-        <v>4007</v>
+        <v>4009</v>
       </c>
       <c r="I903" s="0" t="s">
-        <v>4008</v>
+        <v>4010</v>
       </c>
       <c r="J903" s="0" t="s">
         <v>35</v>
@@ -59156,19 +59192,19 @@
         <v>2207</v>
       </c>
       <c r="E904" s="0" t="s">
-        <v>4009</v>
+        <v>4011</v>
       </c>
       <c r="F904" s="0" t="s">
-        <v>4010</v>
+        <v>4012</v>
       </c>
       <c r="G904" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H904" s="0" t="s">
-        <v>4011</v>
+        <v>4013</v>
       </c>
       <c r="I904" s="0" t="s">
-        <v>4012</v>
+        <v>4014</v>
       </c>
       <c r="J904" s="0" t="s">
         <v>181</v>
@@ -59212,10 +59248,10 @@
         <v>94</v>
       </c>
       <c r="H905" s="0" t="s">
-        <v>4013</v>
+        <v>4015</v>
       </c>
       <c r="I905" s="0" t="s">
-        <v>4014</v>
+        <v>4016</v>
       </c>
       <c r="J905" s="0" t="s">
         <v>123</v>
@@ -59277,7 +59313,7 @@
         <v>38</v>
       </c>
       <c r="P906" s="0" t="s">
-        <v>4015</v>
+        <v>4017</v>
       </c>
       <c r="R906" s="0" t="s">
         <v>748</v>
@@ -59306,10 +59342,10 @@
         <v>94</v>
       </c>
       <c r="H907" s="0" t="s">
-        <v>4016</v>
+        <v>4018</v>
       </c>
       <c r="I907" s="0" t="s">
-        <v>4017</v>
+        <v>4019</v>
       </c>
       <c r="J907" s="0" t="s">
         <v>249</v>
@@ -59388,7 +59424,7 @@
         <v>91</v>
       </c>
       <c r="D909" s="0" t="s">
-        <v>3981</v>
+        <v>3983</v>
       </c>
       <c r="E909" s="0" t="s">
         <v>743</v>
@@ -59400,10 +59436,10 @@
         <v>94</v>
       </c>
       <c r="H909" s="0" t="s">
-        <v>4018</v>
+        <v>4020</v>
       </c>
       <c r="I909" s="0" t="s">
-        <v>4019</v>
+        <v>4021</v>
       </c>
       <c r="J909" s="0" t="s">
         <v>3089</v>
@@ -59412,16 +59448,16 @@
         <v>50</v>
       </c>
       <c r="L909" s="0" t="s">
-        <v>3978</v>
+        <v>3980</v>
       </c>
       <c r="O909" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P909" s="0" t="s">
-        <v>3979</v>
+        <v>3981</v>
       </c>
       <c r="R909" s="0" t="s">
-        <v>3980</v>
+        <v>3982</v>
       </c>
     </row>
     <row r="910">
@@ -59435,7 +59471,7 @@
         <v>91</v>
       </c>
       <c r="D910" s="0" t="s">
-        <v>3992</v>
+        <v>3994</v>
       </c>
       <c r="E910" s="0" t="s">
         <v>685</v>
@@ -59447,10 +59483,10 @@
         <v>94</v>
       </c>
       <c r="H910" s="0" t="s">
-        <v>4020</v>
+        <v>4022</v>
       </c>
       <c r="I910" s="0" t="s">
-        <v>4021</v>
+        <v>4023</v>
       </c>
       <c r="J910" s="0" t="s">
         <v>86</v>
@@ -59465,7 +59501,7 @@
         <v>38</v>
       </c>
       <c r="P910" s="0" t="s">
-        <v>3991</v>
+        <v>3993</v>
       </c>
       <c r="R910" s="0" t="s">
         <v>3698</v>
@@ -59494,10 +59530,10 @@
         <v>94</v>
       </c>
       <c r="H911" s="0" t="s">
-        <v>4022</v>
+        <v>4024</v>
       </c>
       <c r="I911" s="0" t="s">
-        <v>4023</v>
+        <v>4025</v>
       </c>
       <c r="J911" s="0" t="s">
         <v>108</v>
@@ -59541,10 +59577,10 @@
         <v>94</v>
       </c>
       <c r="H912" s="0" t="s">
-        <v>4024</v>
+        <v>4026</v>
       </c>
       <c r="I912" s="0" t="s">
-        <v>4025</v>
+        <v>4027</v>
       </c>
       <c r="J912" s="0" t="s">
         <v>123</v>
@@ -59591,7 +59627,7 @@
         <v>750</v>
       </c>
       <c r="I913" s="0" t="s">
-        <v>4026</v>
+        <v>4028</v>
       </c>
       <c r="J913" s="0" t="s">
         <v>746</v>
@@ -59606,7 +59642,7 @@
         <v>38</v>
       </c>
       <c r="P913" s="0" t="s">
-        <v>4015</v>
+        <v>4017</v>
       </c>
       <c r="R913" s="0" t="s">
         <v>748</v>
@@ -59635,10 +59671,10 @@
         <v>94</v>
       </c>
       <c r="H914" s="0" t="s">
-        <v>4027</v>
+        <v>4029</v>
       </c>
       <c r="I914" s="0" t="s">
-        <v>4028</v>
+        <v>4030</v>
       </c>
       <c r="J914" s="0" t="s">
         <v>249</v>
@@ -59670,7 +59706,7 @@
         <v>91</v>
       </c>
       <c r="D915" s="0" t="s">
-        <v>4029</v>
+        <v>4031</v>
       </c>
       <c r="E915" s="0" t="s">
         <v>196</v>
@@ -59682,10 +59718,10 @@
         <v>94</v>
       </c>
       <c r="H915" s="0" t="s">
-        <v>4030</v>
+        <v>4032</v>
       </c>
       <c r="I915" s="0" t="s">
-        <v>4031</v>
+        <v>4033</v>
       </c>
       <c r="J915" s="0" t="s">
         <v>209</v>
@@ -59700,10 +59736,10 @@
         <v>38</v>
       </c>
       <c r="P915" s="0" t="s">
-        <v>4032</v>
+        <v>4034</v>
       </c>
       <c r="R915" s="0" t="s">
-        <v>4033</v>
+        <v>4035</v>
       </c>
     </row>
     <row r="916">
@@ -59717,22 +59753,22 @@
         <v>91</v>
       </c>
       <c r="D916" s="0" t="s">
-        <v>4034</v>
+        <v>4036</v>
       </c>
       <c r="E916" s="0" t="s">
         <v>196</v>
       </c>
       <c r="F916" s="0" t="s">
-        <v>4035</v>
+        <v>4037</v>
       </c>
       <c r="G916" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H916" s="0" t="s">
-        <v>4036</v>
+        <v>4038</v>
       </c>
       <c r="I916" s="0" t="s">
-        <v>4037</v>
+        <v>4039</v>
       </c>
       <c r="J916" s="0" t="s">
         <v>2064</v>
@@ -59747,10 +59783,10 @@
         <v>38</v>
       </c>
       <c r="P916" s="0" t="s">
-        <v>4038</v>
+        <v>4040</v>
       </c>
       <c r="R916" s="0" t="s">
-        <v>4039</v>
+        <v>4041</v>
       </c>
     </row>
     <row r="917">
@@ -59764,7 +59800,7 @@
         <v>91</v>
       </c>
       <c r="D917" s="0" t="s">
-        <v>4040</v>
+        <v>4042</v>
       </c>
       <c r="E917" s="0" t="s">
         <v>196</v>
@@ -59776,10 +59812,10 @@
         <v>94</v>
       </c>
       <c r="H917" s="0" t="s">
-        <v>4041</v>
+        <v>4043</v>
       </c>
       <c r="I917" s="0" t="s">
-        <v>4042</v>
+        <v>4044</v>
       </c>
       <c r="J917" s="0" t="s">
         <v>375</v>
@@ -59794,10 +59830,10 @@
         <v>38</v>
       </c>
       <c r="P917" s="0" t="s">
-        <v>4043</v>
+        <v>4045</v>
       </c>
       <c r="R917" s="0" t="s">
-        <v>4044</v>
+        <v>4046</v>
       </c>
     </row>
     <row r="918">
@@ -59811,22 +59847,22 @@
         <v>91</v>
       </c>
       <c r="D918" s="0" t="s">
-        <v>4045</v>
+        <v>4047</v>
       </c>
       <c r="E918" s="0" t="s">
         <v>196</v>
       </c>
       <c r="F918" s="0" t="s">
-        <v>4046</v>
+        <v>4048</v>
       </c>
       <c r="G918" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H918" s="0" t="s">
-        <v>4047</v>
+        <v>4049</v>
       </c>
       <c r="I918" s="0" t="s">
-        <v>4048</v>
+        <v>4050</v>
       </c>
       <c r="J918" s="0" t="s">
         <v>1034</v>
@@ -59841,10 +59877,10 @@
         <v>38</v>
       </c>
       <c r="P918" s="0" t="s">
-        <v>4049</v>
+        <v>4051</v>
       </c>
       <c r="R918" s="0" t="s">
-        <v>4050</v>
+        <v>4052</v>
       </c>
     </row>
     <row r="919">
@@ -59858,22 +59894,22 @@
         <v>91</v>
       </c>
       <c r="D919" s="0" t="s">
-        <v>4051</v>
+        <v>4053</v>
       </c>
       <c r="E919" s="0" t="s">
         <v>214</v>
       </c>
       <c r="F919" s="0" t="s">
-        <v>4052</v>
+        <v>4054</v>
       </c>
       <c r="G919" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H919" s="0" t="s">
-        <v>4053</v>
+        <v>4055</v>
       </c>
       <c r="I919" s="0" t="s">
-        <v>4054</v>
+        <v>4056</v>
       </c>
       <c r="J919" s="0" t="s">
         <v>784</v>
@@ -59888,10 +59924,10 @@
         <v>51</v>
       </c>
       <c r="P919" s="0" t="s">
-        <v>4055</v>
+        <v>4057</v>
       </c>
       <c r="R919" s="0" t="s">
-        <v>4056</v>
+        <v>4058</v>
       </c>
     </row>
     <row r="920">
@@ -59905,7 +59941,7 @@
         <v>91</v>
       </c>
       <c r="D920" s="0" t="s">
-        <v>4057</v>
+        <v>4059</v>
       </c>
       <c r="E920" s="0" t="s">
         <v>196</v>
@@ -59917,10 +59953,10 @@
         <v>94</v>
       </c>
       <c r="H920" s="0" t="s">
-        <v>4058</v>
+        <v>4060</v>
       </c>
       <c r="I920" s="0" t="s">
-        <v>4059</v>
+        <v>4061</v>
       </c>
       <c r="J920" s="0" t="s">
         <v>1034</v>
@@ -59935,10 +59971,10 @@
         <v>38</v>
       </c>
       <c r="P920" s="0" t="s">
-        <v>4060</v>
+        <v>4062</v>
       </c>
       <c r="R920" s="0" t="s">
-        <v>4061</v>
+        <v>4063</v>
       </c>
     </row>
     <row r="921">
@@ -59949,25 +59985,25 @@
         <v>46203.65469700231</v>
       </c>
       <c r="C921" s="0" t="s">
-        <v>3736</v>
+        <v>3738</v>
       </c>
       <c r="D921" s="0" t="s">
-        <v>4062</v>
+        <v>4064</v>
       </c>
       <c r="E921" s="0" t="s">
-        <v>4063</v>
+        <v>4065</v>
       </c>
       <c r="F921" s="0" t="s">
-        <v>4063</v>
+        <v>4065</v>
       </c>
       <c r="G921" s="0" t="s">
-        <v>3739</v>
+        <v>3741</v>
       </c>
       <c r="H921" s="0" t="s">
-        <v>4064</v>
+        <v>4066</v>
       </c>
       <c r="I921" s="0" t="s">
-        <v>4065</v>
+        <v>4067</v>
       </c>
       <c r="J921" s="0" t="s">
         <v>3683</v>
@@ -59982,7 +60018,7 @@
         <v>38</v>
       </c>
       <c r="V921" s="0" t="s">
-        <v>4066</v>
+        <v>4068</v>
       </c>
     </row>
     <row r="922">
@@ -59996,7 +60032,7 @@
         <v>2738</v>
       </c>
       <c r="D922" s="0" t="s">
-        <v>4067</v>
+        <v>4069</v>
       </c>
       <c r="E922" s="0" t="s">
         <v>30</v>
@@ -60008,10 +60044,10 @@
         <v>2741</v>
       </c>
       <c r="H922" s="0" t="s">
-        <v>4068</v>
+        <v>4070</v>
       </c>
       <c r="I922" s="0" t="s">
-        <v>4069</v>
+        <v>4071</v>
       </c>
       <c r="J922" s="0" t="s">
         <v>3089</v>
@@ -60032,7 +60068,7 @@
         <v>3494</v>
       </c>
       <c r="S922" s="0" t="s">
-        <v>4070</v>
+        <v>4072</v>
       </c>
     </row>
     <row r="923">
@@ -60046,7 +60082,7 @@
         <v>2738</v>
       </c>
       <c r="D923" s="0" t="s">
-        <v>4070</v>
+        <v>4072</v>
       </c>
       <c r="E923" s="0" t="s">
         <v>2585</v>
@@ -60058,10 +60094,10 @@
         <v>2741</v>
       </c>
       <c r="H923" s="0" t="s">
-        <v>4071</v>
+        <v>4073</v>
       </c>
       <c r="I923" s="0" t="s">
-        <v>4072</v>
+        <v>4074</v>
       </c>
       <c r="J923" s="0" t="s">
         <v>150</v>
@@ -60093,22 +60129,22 @@
         <v>28</v>
       </c>
       <c r="D924" s="0" t="s">
-        <v>4073</v>
+        <v>4075</v>
       </c>
       <c r="E924" s="0" t="s">
         <v>76</v>
       </c>
       <c r="F924" s="0" t="s">
-        <v>4074</v>
+        <v>4076</v>
       </c>
       <c r="G924" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H924" s="0" t="s">
-        <v>4075</v>
+        <v>4077</v>
       </c>
       <c r="I924" s="0" t="s">
-        <v>4076</v>
+        <v>4078</v>
       </c>
       <c r="J924" s="0" t="s">
         <v>329</v>
@@ -60123,10 +60159,10 @@
         <v>38</v>
       </c>
       <c r="R924" s="0" t="s">
-        <v>4077</v>
+        <v>4079</v>
       </c>
       <c r="S924" s="0" t="s">
-        <v>4078</v>
+        <v>4080</v>
       </c>
     </row>
     <row r="925">
@@ -60140,7 +60176,7 @@
         <v>28</v>
       </c>
       <c r="D925" s="0" t="s">
-        <v>4078</v>
+        <v>4080</v>
       </c>
       <c r="E925" s="0" t="s">
         <v>66</v>
@@ -60152,10 +60188,10 @@
         <v>32</v>
       </c>
       <c r="H925" s="0" t="s">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="I925" s="0" t="s">
-        <v>4080</v>
+        <v>4082</v>
       </c>
       <c r="J925" s="0" t="s">
         <v>746</v>
@@ -60170,7 +60206,7 @@
         <v>38</v>
       </c>
       <c r="R925" s="0" t="s">
-        <v>4077</v>
+        <v>4079</v>
       </c>
     </row>
     <row r="926">
@@ -60184,22 +60220,22 @@
         <v>2720</v>
       </c>
       <c r="D926" s="0" t="s">
-        <v>4081</v>
+        <v>4083</v>
       </c>
       <c r="E926" s="0" t="s">
-        <v>4082</v>
+        <v>4084</v>
       </c>
       <c r="F926" s="0" t="s">
-        <v>4082</v>
+        <v>4084</v>
       </c>
       <c r="G926" s="0" t="s">
         <v>2720</v>
       </c>
       <c r="H926" s="0" t="s">
-        <v>4083</v>
+        <v>4085</v>
       </c>
       <c r="I926" s="0" t="s">
-        <v>4084</v>
+        <v>4086</v>
       </c>
       <c r="J926" s="0" t="s">
         <v>473</v>
@@ -60208,13 +60244,13 @@
         <v>2230</v>
       </c>
       <c r="L926" s="0" t="s">
-        <v>4085</v>
+        <v>4087</v>
       </c>
       <c r="O926" s="0" t="s">
         <v>38</v>
       </c>
       <c r="R926" s="0" t="s">
-        <v>4086</v>
+        <v>4088</v>
       </c>
     </row>
     <row r="927">
@@ -60228,7 +60264,7 @@
         <v>28</v>
       </c>
       <c r="D927" s="0" t="s">
-        <v>4087</v>
+        <v>4089</v>
       </c>
       <c r="E927" s="0" t="s">
         <v>104</v>
@@ -60240,10 +60276,10 @@
         <v>32</v>
       </c>
       <c r="H927" s="0" t="s">
-        <v>4088</v>
+        <v>4090</v>
       </c>
       <c r="I927" s="0" t="s">
-        <v>4089</v>
+        <v>4091</v>
       </c>
       <c r="J927" s="0" t="s">
         <v>86</v>
@@ -60258,10 +60294,10 @@
         <v>38</v>
       </c>
       <c r="P927" s="0" t="s">
-        <v>4090</v>
+        <v>4092</v>
       </c>
       <c r="R927" s="0" t="s">
-        <v>4091</v>
+        <v>4093</v>
       </c>
     </row>
     <row r="928">
@@ -60275,7 +60311,7 @@
         <v>28</v>
       </c>
       <c r="D928" s="0" t="s">
-        <v>4092</v>
+        <v>4094</v>
       </c>
       <c r="E928" s="0" t="s">
         <v>104</v>
@@ -60287,10 +60323,10 @@
         <v>32</v>
       </c>
       <c r="H928" s="0" t="s">
-        <v>4093</v>
+        <v>4095</v>
       </c>
       <c r="I928" s="0" t="s">
-        <v>4094</v>
+        <v>4096</v>
       </c>
       <c r="J928" s="0" t="s">
         <v>86</v>
@@ -60305,10 +60341,10 @@
         <v>38</v>
       </c>
       <c r="P928" s="0" t="s">
-        <v>4090</v>
+        <v>4092</v>
       </c>
       <c r="R928" s="0" t="s">
-        <v>4091</v>
+        <v>4093</v>
       </c>
     </row>
     <row r="929">
@@ -60322,7 +60358,7 @@
         <v>28</v>
       </c>
       <c r="D929" s="0" t="s">
-        <v>4095</v>
+        <v>4097</v>
       </c>
       <c r="E929" s="0" t="s">
         <v>60</v>
@@ -60334,10 +60370,10 @@
         <v>32</v>
       </c>
       <c r="H929" s="0" t="s">
-        <v>4096</v>
+        <v>4098</v>
       </c>
       <c r="I929" s="0" t="s">
-        <v>4097</v>
+        <v>4099</v>
       </c>
       <c r="J929" s="0" t="s">
         <v>1973</v>
@@ -60352,16 +60388,16 @@
         <v>38</v>
       </c>
       <c r="P929" s="0" t="s">
-        <v>4090</v>
+        <v>4092</v>
       </c>
       <c r="R929" s="0" t="s">
-        <v>4091</v>
+        <v>4093</v>
       </c>
       <c r="S929" s="0" t="s">
-        <v>4087</v>
+        <v>4089</v>
       </c>
       <c r="T929" s="0" t="s">
-        <v>4092</v>
+        <v>4094</v>
       </c>
     </row>
     <row r="930">
@@ -60375,22 +60411,22 @@
         <v>28</v>
       </c>
       <c r="D930" s="0" t="s">
-        <v>4098</v>
+        <v>4100</v>
       </c>
       <c r="E930" s="0" t="s">
         <v>60</v>
       </c>
       <c r="F930" s="0" t="s">
-        <v>4099</v>
+        <v>4101</v>
       </c>
       <c r="G930" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H930" s="0" t="s">
-        <v>4100</v>
+        <v>4102</v>
       </c>
       <c r="I930" s="0" t="s">
-        <v>4101</v>
+        <v>4103</v>
       </c>
       <c r="J930" s="0" t="s">
         <v>108</v>
@@ -60425,22 +60461,22 @@
         <v>28</v>
       </c>
       <c r="D931" s="0" t="s">
-        <v>4102</v>
+        <v>4104</v>
       </c>
       <c r="E931" s="0" t="s">
         <v>231</v>
       </c>
       <c r="F931" s="0" t="s">
-        <v>4103</v>
+        <v>4105</v>
       </c>
       <c r="G931" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H931" s="0" t="s">
-        <v>4104</v>
+        <v>4106</v>
       </c>
       <c r="I931" s="0" t="s">
-        <v>4105</v>
+        <v>4107</v>
       </c>
       <c r="J931" s="0" t="s">
         <v>80</v>
@@ -60455,10 +60491,10 @@
         <v>38</v>
       </c>
       <c r="P931" s="0" t="s">
-        <v>4106</v>
+        <v>4108</v>
       </c>
       <c r="R931" s="0" t="s">
-        <v>4107</v>
+        <v>4109</v>
       </c>
     </row>
     <row r="932">
@@ -60472,22 +60508,22 @@
         <v>91</v>
       </c>
       <c r="D932" s="0" t="s">
-        <v>4108</v>
+        <v>4110</v>
       </c>
       <c r="E932" s="0" t="s">
-        <v>4109</v>
+        <v>4111</v>
       </c>
       <c r="F932" s="0" t="s">
-        <v>4110</v>
+        <v>4112</v>
       </c>
       <c r="G932" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H932" s="0" t="s">
-        <v>4111</v>
+        <v>4113</v>
       </c>
       <c r="I932" s="0" t="s">
-        <v>4112</v>
+        <v>4114</v>
       </c>
       <c r="J932" s="0" t="s">
         <v>304</v>
@@ -60502,10 +60538,10 @@
         <v>38</v>
       </c>
       <c r="P932" s="0" t="s">
-        <v>4113</v>
+        <v>4115</v>
       </c>
       <c r="R932" s="0" t="s">
-        <v>4114</v>
+        <v>4116</v>
       </c>
     </row>
     <row r="933">
@@ -60519,7 +60555,7 @@
         <v>91</v>
       </c>
       <c r="D933" s="0" t="s">
-        <v>4115</v>
+        <v>4117</v>
       </c>
       <c r="E933" s="0" t="s">
         <v>76</v>
@@ -60531,10 +60567,10 @@
         <v>94</v>
       </c>
       <c r="H933" s="0" t="s">
-        <v>4116</v>
+        <v>4118</v>
       </c>
       <c r="I933" s="0" t="s">
-        <v>4117</v>
+        <v>4119</v>
       </c>
       <c r="J933" s="0" t="s">
         <v>1034</v>
@@ -60549,13 +60585,13 @@
         <v>38</v>
       </c>
       <c r="P933" s="0" t="s">
-        <v>4118</v>
+        <v>4120</v>
       </c>
       <c r="R933" s="0" t="s">
-        <v>4119</v>
+        <v>4121</v>
       </c>
       <c r="S933" s="0" t="s">
-        <v>4120</v>
+        <v>4122</v>
       </c>
       <c r="T933" s="0" t="s">
         <v>52</v>
@@ -60572,7 +60608,7 @@
         <v>91</v>
       </c>
       <c r="D934" s="0" t="s">
-        <v>4121</v>
+        <v>4123</v>
       </c>
       <c r="E934" s="0" t="s">
         <v>76</v>
@@ -60584,10 +60620,10 @@
         <v>94</v>
       </c>
       <c r="H934" s="0" t="s">
-        <v>4122</v>
+        <v>4124</v>
       </c>
       <c r="I934" s="0" t="s">
-        <v>4123</v>
+        <v>4125</v>
       </c>
       <c r="J934" s="0" t="s">
         <v>897</v>
@@ -60602,16 +60638,16 @@
         <v>38</v>
       </c>
       <c r="P934" s="0" t="s">
-        <v>4124</v>
+        <v>4126</v>
       </c>
       <c r="R934" s="0" t="s">
-        <v>4125</v>
+        <v>4127</v>
       </c>
       <c r="S934" s="0" t="s">
-        <v>4126</v>
+        <v>4128</v>
       </c>
       <c r="T934" s="0" t="s">
-        <v>4127</v>
+        <v>4129</v>
       </c>
     </row>
     <row r="935">
@@ -60625,7 +60661,7 @@
         <v>91</v>
       </c>
       <c r="D935" s="0" t="s">
-        <v>4126</v>
+        <v>4128</v>
       </c>
       <c r="E935" s="0" t="s">
         <v>759</v>
@@ -60637,10 +60673,10 @@
         <v>94</v>
       </c>
       <c r="H935" s="0" t="s">
-        <v>4128</v>
+        <v>4130</v>
       </c>
       <c r="I935" s="0" t="s">
-        <v>4129</v>
+        <v>4131</v>
       </c>
       <c r="J935" s="0" t="s">
         <v>454</v>
@@ -60655,10 +60691,10 @@
         <v>38</v>
       </c>
       <c r="P935" s="0" t="s">
-        <v>4124</v>
+        <v>4126</v>
       </c>
       <c r="R935" s="0" t="s">
-        <v>4125</v>
+        <v>4127</v>
       </c>
     </row>
     <row r="936">
@@ -60672,7 +60708,7 @@
         <v>91</v>
       </c>
       <c r="D936" s="0" t="s">
-        <v>4127</v>
+        <v>4129</v>
       </c>
       <c r="E936" s="0" t="s">
         <v>759</v>
@@ -60684,10 +60720,10 @@
         <v>94</v>
       </c>
       <c r="H936" s="0" t="s">
-        <v>4130</v>
+        <v>4132</v>
       </c>
       <c r="I936" s="0" t="s">
-        <v>4131</v>
+        <v>4133</v>
       </c>
       <c r="J936" s="0" t="s">
         <v>454</v>
@@ -60702,10 +60738,10 @@
         <v>38</v>
       </c>
       <c r="P936" s="0" t="s">
-        <v>4124</v>
+        <v>4126</v>
       </c>
       <c r="R936" s="0" t="s">
-        <v>4125</v>
+        <v>4127</v>
       </c>
     </row>
     <row r="937">
@@ -60719,7 +60755,7 @@
         <v>91</v>
       </c>
       <c r="D937" s="0" t="s">
-        <v>4120</v>
+        <v>4122</v>
       </c>
       <c r="E937" s="0" t="s">
         <v>2585</v>
@@ -60731,10 +60767,10 @@
         <v>94</v>
       </c>
       <c r="H937" s="0" t="s">
-        <v>4132</v>
+        <v>4134</v>
       </c>
       <c r="I937" s="0" t="s">
-        <v>4133</v>
+        <v>4135</v>
       </c>
       <c r="J937" s="0" t="s">
         <v>403</v>
@@ -60749,10 +60785,10 @@
         <v>38</v>
       </c>
       <c r="P937" s="0" t="s">
-        <v>4118</v>
+        <v>4120</v>
       </c>
       <c r="R937" s="0" t="s">
-        <v>4119</v>
+        <v>4121</v>
       </c>
     </row>
     <row r="938">
@@ -60778,10 +60814,10 @@
         <v>94</v>
       </c>
       <c r="H938" s="0" t="s">
-        <v>4134</v>
+        <v>4136</v>
       </c>
       <c r="I938" s="0" t="s">
-        <v>4135</v>
+        <v>4137</v>
       </c>
       <c r="J938" s="0" t="s">
         <v>519</v>
@@ -60813,7 +60849,7 @@
         <v>128</v>
       </c>
       <c r="D939" s="0" t="s">
-        <v>4136</v>
+        <v>4138</v>
       </c>
       <c r="E939" s="0" t="s">
         <v>60</v>
@@ -60825,10 +60861,10 @@
         <v>1887</v>
       </c>
       <c r="H939" s="0" t="s">
-        <v>4137</v>
+        <v>4139</v>
       </c>
       <c r="I939" s="0" t="s">
-        <v>4138</v>
+        <v>4140</v>
       </c>
       <c r="J939" s="0" t="s">
         <v>86</v>
@@ -60863,7 +60899,7 @@
         <v>91</v>
       </c>
       <c r="D940" s="0" t="s">
-        <v>4139</v>
+        <v>4141</v>
       </c>
       <c r="E940" s="0" t="s">
         <v>1038</v>
@@ -60875,10 +60911,10 @@
         <v>94</v>
       </c>
       <c r="H940" s="0" t="s">
-        <v>4140</v>
+        <v>4142</v>
       </c>
       <c r="I940" s="0" t="s">
-        <v>4141</v>
+        <v>4143</v>
       </c>
       <c r="J940" s="0" t="s">
         <v>403</v>
@@ -60896,7 +60932,7 @@
         <v>3634</v>
       </c>
       <c r="R940" s="0" t="s">
-        <v>4142</v>
+        <v>4144</v>
       </c>
     </row>
     <row r="941">
@@ -60910,22 +60946,22 @@
         <v>954</v>
       </c>
       <c r="D941" s="0" t="s">
-        <v>4143</v>
+        <v>4145</v>
       </c>
       <c r="E941" s="0" t="s">
-        <v>4144</v>
+        <v>4146</v>
       </c>
       <c r="F941" s="0" t="s">
-        <v>4145</v>
+        <v>4147</v>
       </c>
       <c r="G941" s="0" t="s">
         <v>954</v>
       </c>
       <c r="H941" s="0" t="s">
-        <v>4146</v>
+        <v>4148</v>
       </c>
       <c r="I941" s="0" t="s">
-        <v>4147</v>
+        <v>4149</v>
       </c>
       <c r="J941" s="0" t="s">
         <v>423</v>
@@ -60940,10 +60976,10 @@
         <v>38</v>
       </c>
       <c r="P941" s="0" t="s">
-        <v>4148</v>
+        <v>4150</v>
       </c>
       <c r="R941" s="0" t="s">
-        <v>4149</v>
+        <v>4151</v>
       </c>
       <c r="S941" s="0" t="s">
         <v>1052</v>
@@ -60963,22 +60999,22 @@
         <v>2720</v>
       </c>
       <c r="D942" s="0" t="s">
-        <v>4150</v>
+        <v>4152</v>
       </c>
       <c r="E942" s="0" t="s">
-        <v>4151</v>
+        <v>4153</v>
       </c>
       <c r="F942" s="0" t="s">
-        <v>4152</v>
+        <v>4154</v>
       </c>
       <c r="G942" s="0" t="s">
-        <v>4153</v>
+        <v>4155</v>
       </c>
       <c r="H942" s="0" t="s">
-        <v>4154</v>
+        <v>4156</v>
       </c>
       <c r="I942" s="0" t="s">
-        <v>4155</v>
+        <v>4157</v>
       </c>
       <c r="J942" s="0" t="s">
         <v>473</v>
@@ -60993,7 +61029,7 @@
         <v>38</v>
       </c>
       <c r="R942" s="0" t="s">
-        <v>4156</v>
+        <v>4158</v>
       </c>
     </row>
     <row r="943">
@@ -61007,7 +61043,7 @@
         <v>128</v>
       </c>
       <c r="D943" s="0" t="s">
-        <v>4157</v>
+        <v>4159</v>
       </c>
       <c r="E943" s="0" t="s">
         <v>1293</v>
@@ -61019,10 +61055,10 @@
         <v>131</v>
       </c>
       <c r="H943" s="0" t="s">
-        <v>4158</v>
+        <v>4160</v>
       </c>
       <c r="I943" s="0" t="s">
-        <v>4159</v>
+        <v>4161</v>
       </c>
       <c r="J943" s="0" t="s">
         <v>444</v>
@@ -61031,16 +61067,16 @@
         <v>161</v>
       </c>
       <c r="L943" s="0" t="s">
-        <v>4160</v>
+        <v>4162</v>
       </c>
       <c r="O943" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P943" s="0" t="s">
-        <v>4161</v>
+        <v>4163</v>
       </c>
       <c r="R943" s="0" t="s">
-        <v>4162</v>
+        <v>4164</v>
       </c>
       <c r="S943" s="0" t="s">
         <v>1001</v>
@@ -61057,7 +61093,7 @@
         <v>91</v>
       </c>
       <c r="D944" s="0" t="s">
-        <v>4163</v>
+        <v>4165</v>
       </c>
       <c r="E944" s="0" t="s">
         <v>60</v>
@@ -61069,10 +61105,10 @@
         <v>94</v>
       </c>
       <c r="H944" s="0" t="s">
-        <v>4164</v>
+        <v>4166</v>
       </c>
       <c r="I944" s="0" t="s">
-        <v>4165</v>
+        <v>4167</v>
       </c>
       <c r="J944" s="0" t="s">
         <v>218</v>
@@ -61087,13 +61123,13 @@
         <v>38</v>
       </c>
       <c r="P944" s="0" t="s">
-        <v>4166</v>
+        <v>4168</v>
       </c>
       <c r="R944" s="0" t="s">
-        <v>4167</v>
+        <v>4169</v>
       </c>
       <c r="S944" s="0" t="s">
-        <v>4168</v>
+        <v>4170</v>
       </c>
     </row>
     <row r="945">
@@ -61107,7 +61143,7 @@
         <v>91</v>
       </c>
       <c r="D945" s="0" t="s">
-        <v>4168</v>
+        <v>4170</v>
       </c>
       <c r="E945" s="0" t="s">
         <v>759</v>
@@ -61119,10 +61155,10 @@
         <v>94</v>
       </c>
       <c r="H945" s="0" t="s">
-        <v>4169</v>
+        <v>4171</v>
       </c>
       <c r="I945" s="0" t="s">
-        <v>4170</v>
+        <v>4172</v>
       </c>
       <c r="J945" s="0" t="s">
         <v>1801</v>
@@ -61137,10 +61173,10 @@
         <v>38</v>
       </c>
       <c r="P945" s="0" t="s">
-        <v>4166</v>
+        <v>4168</v>
       </c>
       <c r="R945" s="0" t="s">
-        <v>4167</v>
+        <v>4169</v>
       </c>
     </row>
     <row r="946">
@@ -61154,7 +61190,7 @@
         <v>91</v>
       </c>
       <c r="D946" s="0" t="s">
-        <v>4171</v>
+        <v>4173</v>
       </c>
       <c r="E946" s="0" t="s">
         <v>196</v>
@@ -61166,10 +61202,10 @@
         <v>94</v>
       </c>
       <c r="H946" s="0" t="s">
-        <v>4172</v>
+        <v>4174</v>
       </c>
       <c r="I946" s="0" t="s">
-        <v>4173</v>
+        <v>4175</v>
       </c>
       <c r="J946" s="0" t="s">
         <v>535</v>
@@ -61178,19 +61214,19 @@
         <v>87</v>
       </c>
       <c r="L946" s="0" t="s">
-        <v>4174</v>
+        <v>4176</v>
       </c>
       <c r="O946" s="0" t="s">
         <v>51</v>
       </c>
       <c r="P946" s="0" t="s">
-        <v>4175</v>
+        <v>4177</v>
       </c>
       <c r="R946" s="0" t="s">
-        <v>4176</v>
+        <v>4178</v>
       </c>
       <c r="S946" s="0" t="s">
-        <v>4177</v>
+        <v>4179</v>
       </c>
     </row>
     <row r="947">
@@ -61204,7 +61240,7 @@
         <v>91</v>
       </c>
       <c r="D947" s="0" t="s">
-        <v>4177</v>
+        <v>4179</v>
       </c>
       <c r="E947" s="0" t="s">
         <v>759</v>
@@ -61216,10 +61252,10 @@
         <v>94</v>
       </c>
       <c r="H947" s="0" t="s">
-        <v>4178</v>
+        <v>4180</v>
       </c>
       <c r="I947" s="0" t="s">
-        <v>4179</v>
+        <v>4181</v>
       </c>
       <c r="J947" s="0" t="s">
         <v>3072</v>
@@ -61234,10 +61270,10 @@
         <v>38</v>
       </c>
       <c r="P947" s="0" t="s">
-        <v>4175</v>
+        <v>4177</v>
       </c>
       <c r="R947" s="0" t="s">
-        <v>4176</v>
+        <v>4178</v>
       </c>
     </row>
     <row r="948">
@@ -61251,7 +61287,7 @@
         <v>91</v>
       </c>
       <c r="D948" s="0" t="s">
-        <v>4180</v>
+        <v>4182</v>
       </c>
       <c r="E948" s="0" t="s">
         <v>60</v>
@@ -61263,10 +61299,10 @@
         <v>94</v>
       </c>
       <c r="H948" s="0" t="s">
-        <v>4181</v>
+        <v>4183</v>
       </c>
       <c r="I948" s="0" t="s">
-        <v>4182</v>
+        <v>4184</v>
       </c>
       <c r="J948" s="0" t="s">
         <v>300</v>
@@ -61281,16 +61317,16 @@
         <v>38</v>
       </c>
       <c r="P948" s="0" t="s">
-        <v>4183</v>
+        <v>4185</v>
       </c>
       <c r="R948" s="0" t="s">
-        <v>4184</v>
+        <v>4186</v>
       </c>
       <c r="S948" s="0" t="s">
-        <v>4185</v>
+        <v>4187</v>
       </c>
       <c r="T948" s="0" t="s">
-        <v>4186</v>
+        <v>4188</v>
       </c>
     </row>
     <row r="949">
@@ -61304,7 +61340,7 @@
         <v>91</v>
       </c>
       <c r="D949" s="0" t="s">
-        <v>4185</v>
+        <v>4187</v>
       </c>
       <c r="E949" s="0" t="s">
         <v>685</v>
@@ -61316,10 +61352,10 @@
         <v>94</v>
       </c>
       <c r="H949" s="0" t="s">
-        <v>4187</v>
+        <v>4189</v>
       </c>
       <c r="I949" s="0" t="s">
-        <v>4188</v>
+        <v>4190</v>
       </c>
       <c r="J949" s="0" t="s">
         <v>897</v>
@@ -61334,10 +61370,10 @@
         <v>38</v>
       </c>
       <c r="P949" s="0" t="s">
-        <v>4183</v>
+        <v>4185</v>
       </c>
       <c r="R949" s="0" t="s">
-        <v>4184</v>
+        <v>4186</v>
       </c>
     </row>
     <row r="950">
@@ -61351,7 +61387,7 @@
         <v>91</v>
       </c>
       <c r="D950" s="0" t="s">
-        <v>4186</v>
+        <v>4188</v>
       </c>
       <c r="E950" s="0" t="s">
         <v>685</v>
@@ -61363,10 +61399,10 @@
         <v>94</v>
       </c>
       <c r="H950" s="0" t="s">
-        <v>4189</v>
+        <v>4191</v>
       </c>
       <c r="I950" s="0" t="s">
-        <v>4190</v>
+        <v>4192</v>
       </c>
       <c r="J950" s="0" t="s">
         <v>897</v>
@@ -61381,10 +61417,10 @@
         <v>38</v>
       </c>
       <c r="P950" s="0" t="s">
-        <v>4183</v>
+        <v>4185</v>
       </c>
       <c r="R950" s="0" t="s">
-        <v>4184</v>
+        <v>4186</v>
       </c>
     </row>
     <row r="951">
@@ -61410,10 +61446,10 @@
         <v>2663</v>
       </c>
       <c r="H951" s="0" t="s">
-        <v>4191</v>
+        <v>4193</v>
       </c>
       <c r="I951" s="0" t="s">
-        <v>4192</v>
+        <v>4194</v>
       </c>
       <c r="J951" s="0" t="s">
         <v>2668</v>
@@ -61428,7 +61464,7 @@
         <v>38</v>
       </c>
       <c r="V951" s="0" t="s">
-        <v>4193</v>
+        <v>4195</v>
       </c>
     </row>
     <row r="952">
@@ -61442,25 +61478,25 @@
         <v>2663</v>
       </c>
       <c r="D952" s="0" t="s">
-        <v>4194</v>
+        <v>4196</v>
       </c>
       <c r="E952" s="0" t="s">
-        <v>4195</v>
+        <v>4197</v>
       </c>
       <c r="F952" s="0" t="s">
-        <v>4195</v>
+        <v>4197</v>
       </c>
       <c r="G952" s="0" t="s">
         <v>2663</v>
       </c>
       <c r="H952" s="0" t="s">
-        <v>4196</v>
+        <v>4198</v>
       </c>
       <c r="I952" s="0" t="s">
-        <v>4197</v>
+        <v>4199</v>
       </c>
       <c r="J952" s="0" t="s">
-        <v>4198</v>
+        <v>4200</v>
       </c>
       <c r="K952" s="0" t="s">
         <v>201</v>
@@ -61472,7 +61508,7 @@
         <v>38</v>
       </c>
       <c r="R952" s="0" t="s">
-        <v>4193</v>
+        <v>4195</v>
       </c>
     </row>
     <row r="953">
@@ -61486,22 +61522,22 @@
         <v>128</v>
       </c>
       <c r="D953" s="0" t="s">
-        <v>4199</v>
+        <v>4201</v>
       </c>
       <c r="E953" s="0" t="s">
-        <v>4200</v>
+        <v>4202</v>
       </c>
       <c r="F953" s="0" t="s">
-        <v>4200</v>
+        <v>4202</v>
       </c>
       <c r="G953" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H953" s="0" t="s">
-        <v>4201</v>
+        <v>4203</v>
       </c>
       <c r="I953" s="0" t="s">
-        <v>4202</v>
+        <v>4204</v>
       </c>
       <c r="J953" s="0" t="s">
         <v>186</v>
@@ -61539,22 +61575,22 @@
         <v>28</v>
       </c>
       <c r="D954" s="0" t="s">
-        <v>4203</v>
+        <v>4205</v>
       </c>
       <c r="E954" s="0" t="s">
         <v>76</v>
       </c>
       <c r="F954" s="0" t="s">
-        <v>4204</v>
+        <v>4206</v>
       </c>
       <c r="G954" s="0" t="s">
         <v>32</v>
       </c>
       <c r="H954" s="0" t="s">
-        <v>4205</v>
+        <v>4207</v>
       </c>
       <c r="I954" s="0" t="s">
-        <v>4206</v>
+        <v>4208</v>
       </c>
       <c r="J954" s="0" t="s">
         <v>142</v>
@@ -61563,13 +61599,13 @@
         <v>36</v>
       </c>
       <c r="L954" s="0" t="s">
-        <v>4207</v>
+        <v>4209</v>
       </c>
       <c r="O954" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P954" s="0" t="s">
-        <v>4208</v>
+        <v>4210</v>
       </c>
       <c r="R954" s="0" t="s">
         <v>2287</v>
@@ -61592,22 +61628,22 @@
         <v>128</v>
       </c>
       <c r="D955" s="0" t="s">
-        <v>4209</v>
+        <v>4211</v>
       </c>
       <c r="E955" s="0" t="s">
-        <v>4210</v>
+        <v>4212</v>
       </c>
       <c r="F955" s="0" t="s">
-        <v>4210</v>
+        <v>4212</v>
       </c>
       <c r="G955" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H955" s="0" t="s">
-        <v>4211</v>
+        <v>4213</v>
       </c>
       <c r="I955" s="0" t="s">
-        <v>4210</v>
+        <v>4212</v>
       </c>
       <c r="J955" s="0" t="s">
         <v>1114</v>
@@ -61616,19 +61652,19 @@
         <v>71</v>
       </c>
       <c r="L955" s="0" t="s">
-        <v>4212</v>
+        <v>4214</v>
       </c>
       <c r="O955" s="0" t="s">
         <v>38</v>
       </c>
       <c r="R955" s="0" t="s">
-        <v>4213</v>
+        <v>4215</v>
       </c>
       <c r="S955" s="0" t="s">
-        <v>4214</v>
+        <v>4216</v>
       </c>
       <c r="T955" s="0" t="s">
-        <v>4215</v>
+        <v>4217</v>
       </c>
     </row>
     <row r="956">
@@ -61642,7 +61678,7 @@
         <v>128</v>
       </c>
       <c r="D956" s="0" t="s">
-        <v>4214</v>
+        <v>4216</v>
       </c>
       <c r="E956" s="0" t="s">
         <v>1320</v>
@@ -61654,10 +61690,10 @@
         <v>131</v>
       </c>
       <c r="H956" s="0" t="s">
-        <v>4216</v>
+        <v>4218</v>
       </c>
       <c r="I956" s="0" t="s">
-        <v>4217</v>
+        <v>4219</v>
       </c>
       <c r="J956" s="0" t="s">
         <v>423</v>
@@ -61666,7 +61702,7 @@
         <v>161</v>
       </c>
       <c r="L956" s="0" t="s">
-        <v>4218</v>
+        <v>4220</v>
       </c>
       <c r="O956" s="0" t="s">
         <v>38</v>
@@ -61683,7 +61719,7 @@
         <v>128</v>
       </c>
       <c r="D957" s="0" t="s">
-        <v>4215</v>
+        <v>4217</v>
       </c>
       <c r="E957" s="0" t="s">
         <v>1320</v>
@@ -61695,10 +61731,10 @@
         <v>131</v>
       </c>
       <c r="H957" s="0" t="s">
-        <v>4219</v>
+        <v>4221</v>
       </c>
       <c r="I957" s="0" t="s">
-        <v>4220</v>
+        <v>4222</v>
       </c>
       <c r="J957" s="0" t="s">
         <v>423</v>
@@ -61707,7 +61743,7 @@
         <v>161</v>
       </c>
       <c r="L957" s="0" t="s">
-        <v>4218</v>
+        <v>4220</v>
       </c>
       <c r="O957" s="0" t="s">
         <v>38</v>
@@ -61724,7 +61760,7 @@
         <v>28</v>
       </c>
       <c r="D958" s="0" t="s">
-        <v>3789</v>
+        <v>3791</v>
       </c>
       <c r="E958" s="0" t="s">
         <v>759</v>
@@ -61736,10 +61772,10 @@
         <v>32</v>
       </c>
       <c r="H958" s="0" t="s">
-        <v>4221</v>
+        <v>4223</v>
       </c>
       <c r="I958" s="0" t="s">
-        <v>4222</v>
+        <v>4224</v>
       </c>
       <c r="J958" s="0" t="s">
         <v>142</v>
@@ -61748,13 +61784,13 @@
         <v>36</v>
       </c>
       <c r="L958" s="0" t="s">
-        <v>3849</v>
+        <v>3851</v>
       </c>
       <c r="O958" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P958" s="0" t="s">
-        <v>3788</v>
+        <v>3790</v>
       </c>
     </row>
     <row r="959">
@@ -61768,7 +61804,7 @@
         <v>28</v>
       </c>
       <c r="D959" s="0" t="s">
-        <v>3790</v>
+        <v>3792</v>
       </c>
       <c r="E959" s="0" t="s">
         <v>759</v>
@@ -61780,10 +61816,10 @@
         <v>32</v>
       </c>
       <c r="H959" s="0" t="s">
-        <v>4223</v>
+        <v>4225</v>
       </c>
       <c r="I959" s="0" t="s">
-        <v>4224</v>
+        <v>4226</v>
       </c>
       <c r="J959" s="0" t="s">
         <v>142</v>
@@ -61792,13 +61828,13 @@
         <v>36</v>
       </c>
       <c r="L959" s="0" t="s">
-        <v>3849</v>
+        <v>3851</v>
       </c>
       <c r="O959" s="0" t="s">
         <v>38</v>
       </c>
       <c r="P959" s="0" t="s">
-        <v>3788</v>
+        <v>3790</v>
       </c>
     </row>
     <row r="960">
@@ -61812,7 +61848,7 @@
         <v>128</v>
       </c>
       <c r="D960" s="0" t="s">
-        <v>4225</v>
+        <v>4227</v>
       </c>
       <c r="E960" s="0" t="s">
         <v>1672</v>
@@ -61824,10 +61860,10 @@
         <v>131</v>
       </c>
       <c r="H960" s="0" t="s">
-        <v>4226</v>
+        <v>4228</v>
       </c>
       <c r="I960" s="0" t="s">
-        <v>4227</v>
+        <v>4229</v>
       </c>
       <c r="J960" s="0" t="s">
         <v>535</v>
@@ -61842,10 +61878,10 @@
         <v>38</v>
       </c>
       <c r="R960" s="0" t="s">
-        <v>4228</v>
+        <v>4230</v>
       </c>
       <c r="S960" s="0" t="s">
-        <v>4229</v>
+        <v>4231</v>
       </c>
     </row>
     <row r="961">
@@ -61859,7 +61895,7 @@
         <v>128</v>
       </c>
       <c r="D961" s="0" t="s">
-        <v>4229</v>
+        <v>4231</v>
       </c>
       <c r="E961" s="0" t="s">
         <v>674</v>
@@ -61871,10 +61907,10 @@
         <v>131</v>
       </c>
       <c r="H961" s="0" t="s">
-        <v>4230</v>
+        <v>4232</v>
       </c>
       <c r="I961" s="0" t="s">
-        <v>4231</v>
+        <v>4233</v>
       </c>
       <c r="J961" s="0" t="s">
         <v>243</v>
@@ -61886,7 +61922,7 @@
         <v>38</v>
       </c>
       <c r="R961" s="0" t="s">
-        <v>4228</v>
+        <v>4230</v>
       </c>
     </row>
     <row r="962">
@@ -61900,7 +61936,7 @@
         <v>128</v>
       </c>
       <c r="D962" s="0" t="s">
-        <v>4232</v>
+        <v>4234</v>
       </c>
       <c r="E962" s="0" t="s">
         <v>1862</v>
@@ -61912,10 +61948,10 @@
         <v>131</v>
       </c>
       <c r="H962" s="0" t="s">
-        <v>4233</v>
+        <v>4235</v>
       </c>
       <c r="I962" s="0" t="s">
-        <v>4234</v>
+        <v>4236</v>
       </c>
       <c r="J962" s="0" t="s">
         <v>108</v>
@@ -61930,10 +61966,10 @@
         <v>38</v>
       </c>
       <c r="R962" s="0" t="s">
-        <v>4235</v>
+        <v>4237</v>
       </c>
       <c r="S962" s="0" t="s">
-        <v>4236</v>
+        <v>4238</v>
       </c>
     </row>
     <row r="963">
@@ -61947,22 +61983,22 @@
         <v>128</v>
       </c>
       <c r="D963" s="0" t="s">
-        <v>4236</v>
+        <v>4238</v>
       </c>
       <c r="E963" s="0" t="s">
-        <v>4237</v>
+        <v>4239</v>
       </c>
       <c r="F963" s="0" t="s">
-        <v>4237</v>
+        <v>4239</v>
       </c>
       <c r="G963" s="0" t="s">
         <v>131</v>
       </c>
       <c r="H963" s="0" t="s">
-        <v>4238</v>
+        <v>4240</v>
       </c>
       <c r="I963" s="0" t="s">
-        <v>4239</v>
+        <v>4241</v>
       </c>
       <c r="J963" s="0" t="s">
         <v>1151</v>
@@ -61977,7 +62013,7 @@
         <v>38</v>
       </c>
       <c r="R963" s="0" t="s">
-        <v>4235</v>
+        <v>4237</v>
       </c>
     </row>
     <row r="964">
@@ -61991,22 +62027,22 @@
         <v>91</v>
       </c>
       <c r="D964" s="0" t="s">
-        <v>4240</v>
+        <v>4242</v>
       </c>
       <c r="E964" s="0" t="s">
         <v>781</v>
       </c>
       <c r="F964" s="0" t="s">
-        <v>4241</v>
+        <v>4243</v>
       </c>
       <c r="G964" s="0" t="s">
         <v>94</v>
       </c>
       <c r="H964" s="0" t="s">
-        <v>4242</v>
+        <v>4244</v>
       </c>
       <c r="I964" s="0" t="s">
-        <v>4243</v>
+        <v>4245</v>
       </c>
       <c r="J964" s="0" t="s">
         <v>70</v>
@@ -62015,16 +62051,16 @@
         <v>36</v>
       </c>
       <c r="L964" s="0" t="s">
-        <v>4244</v>
+        <v>4246</v>
       </c>
       <c r="O964" s="0" t="s">
         <v>38</v>
       </c>
       <c r="R964" s="0" t="s">
-        <v>4176</v>
+        <v>4178</v>
       </c>
       <c r="S964" s="0" t="s">
-        <v>4177</v>
+        <v>4179</v>
       </c>
     </row>
     <row r="965">
@@ -62038,22 +62074,22 @@
         <v>2738</v>
       </c>
       <c r="D965" s="0" t="s">
-        <v>4245</v>
+        <v>4247</v>
       </c>
       <c r="E965" s="0" t="s">
         <v>45</v>
       </c>
       <c r="F965" s="0" t="s">
-        <v>4246</v>
+        <v>4248</v>
       </c>
       <c r="G965" s="0" t="s">
         <v>2741</v>
       </c>
       <c r="H965" s="0" t="s">
-        <v>4247</v>
+        <v>4249</v>
       </c>
       <c r="I965" s="0" t="s">
-        <v>4248</v>
+        <v>4250</v>
       </c>
       <c r="J965" s="0" t="s">
         <v>1141</v>
@@ -62071,7 +62107,7 @@
         <v>3673</v>
       </c>
       <c r="R965" s="0" t="s">
-        <v>4249</v>
+        <v>4251</v>
       </c>
     </row>
     <row r="966">
@@ -62085,7 +62121,7 @@
         <v>28</v>
       </c>
       <c r="D966" s="0" t="s">
-        <v>4250</v>
+        <v>4252</v>
       </c>
       <c r="E966" s="0" t="s">
         <v>165</v>
@@ -62097,13 +62133,13 @@
         <v>147</v>
       </c>
       <c r="H966" s="0" t="s">
-        <v>4251</v>
+        <v>4253</v>
       </c>
       <c r="I966" s="0" t="s">
-        <v>4252</v>
+        <v>4254</v>
       </c>
       <c r="J966" s="0" t="s">
-        <v>4253</v>
+        <v>4255</v>
       </c>
       <c r="K966" s="0" t="s">
         <v>36</v>
@@ -62135,7 +62171,7 @@
         <v>28</v>
       </c>
       <c r="D967" s="0" t="s">
-        <v>4254</v>
+        <v>4256</v>
       </c>
       <c r="E967" s="0" t="s">
         <v>165</v>
@@ -62147,13 +62183,13 @@
         <v>147</v>
       </c>
       <c r="H967" s="0" t="s">
+        <v>4257</v>
+      </c>
+      <c r="I967" s="0" t="s">
+        <v>4258</v>
+      </c>
+      <c r="J967" s="0" t="s">
         <v>4255</v>
-      </c>
-      <c r="I967" s="0" t="s">
-        <v>4256</v>
-      </c>
-      <c r="J967" s="0" t="s">
-        <v>4253</v>
       </c>
       <c r="K967" s="0" t="s">
         <v>36</v>
@@ -62185,7 +62221,7 @@
         <v>954</v>
       </c>
       <c r="D968" s="0" t="s">
-        <v>4257</v>
+        <v>4259</v>
       </c>
       <c r="E968" s="0" t="s">
         <v>781</v>
@@ -62197,10 +62233,10 @@
         <v>954</v>
       </c>
       <c r="H968" s="0" t="s">
-        <v>4258</v>
+        <v>4260</v>
       </c>
       <c r="I968" s="0" t="s">
-        <v>4259</v>
+        <v>4261</v>
       </c>
       <c r="J968" s="0" t="s">
         <v>2064</v>
@@ -62215,7 +62251,7 @@
         <v>38</v>
       </c>
       <c r="R968" s="0" t="s">
-        <v>4260</v>
+        <v>4262</v>
       </c>
     </row>
     <row r="969">
@@ -62229,22 +62265,22 @@
         <v>2720</v>
       </c>
       <c r="D969" s="0" t="s">
-        <v>4261</v>
+        <v>4263</v>
       </c>
       <c r="E969" s="0" t="s">
-        <v>4262</v>
+        <v>4264</v>
       </c>
       <c r="F969" s="0" t="s">
-        <v>4262</v>
+        <v>4264</v>
       </c>
       <c r="G969" s="0" t="s">
         <v>2720</v>
       </c>
       <c r="H969" s="0" t="s">
-        <v>4263</v>
+        <v>4265</v>
       </c>
       <c r="I969" s="0" t="s">
-        <v>4264</v>
+        <v>4266</v>
       </c>
       <c r="J969" s="0" t="s">
         <v>1151</v>
@@ -62259,7 +62295,89 @@
         <v>38</v>
       </c>
       <c r="R969" s="0" t="s">
-        <v>4086</v>
+        <v>4088</v>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" s="0" t="s">
+        <v>3457</v>
+      </c>
+      <c r="B970" s="10">
+        <v>46303.38590450231</v>
+      </c>
+      <c r="C970" s="0" t="s">
+        <v>3686</v>
+      </c>
+      <c r="D970" s="0" t="s">
+        <v>3699</v>
+      </c>
+      <c r="E970" s="0" t="s">
+        <v>3939</v>
+      </c>
+      <c r="F970" s="0" t="s">
+        <v>4267</v>
+      </c>
+      <c r="G970" s="0" t="s">
+        <v>3689</v>
+      </c>
+      <c r="H970" s="0" t="s">
+        <v>4268</v>
+      </c>
+      <c r="I970" s="0" t="s">
+        <v>4269</v>
+      </c>
+      <c r="J970" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="K970" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="L970" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="O970" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" s="0" t="s">
+        <v>3457</v>
+      </c>
+      <c r="B971" s="10">
+        <v>46303.38891412037</v>
+      </c>
+      <c r="C971" s="0" t="s">
+        <v>3686</v>
+      </c>
+      <c r="D971" s="0" t="s">
+        <v>3700</v>
+      </c>
+      <c r="E971" s="0" t="s">
+        <v>4270</v>
+      </c>
+      <c r="F971" s="0" t="s">
+        <v>4270</v>
+      </c>
+      <c r="G971" s="0" t="s">
+        <v>3689</v>
+      </c>
+      <c r="H971" s="0" t="s">
+        <v>4271</v>
+      </c>
+      <c r="I971" s="0" t="s">
+        <v>4272</v>
+      </c>
+      <c r="J971" s="0" t="s">
+        <v>746</v>
+      </c>
+      <c r="K971" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="L971" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="O971" s="0" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados — extração 09/10/2026 09:08 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -20,7 +20,7 @@
     <t>Usuário Geração:</t>
   </si>
   <si>
-    <t>Jadson Rubens Rocha de Oliveira</t>
+    <t>HANNAH MATOS CANESSO MOREIRA</t>
   </si>
   <si>
     <t>Tipo Equipamento</t>
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46303.63243648148</v>
+        <v>46304.38063609954</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 13/10/2026 08:30 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -20,7 +20,7 @@
     <t>Usuário Geração:</t>
   </si>
   <si>
-    <t>HANNAH MATOS CANESSO MOREIRA</t>
+    <t>Jadson Rubens Rocha de Oliveira</t>
   </si>
   <si>
     <t>Tipo Equipamento</t>
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46304.38063609954</v>
+        <v>46308.35485375</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -27210,7 +27210,7 @@
         <v>2</v>
       </c>
       <c r="O264" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P264" s="0" t="s">
         <v>52</v>
@@ -27266,7 +27266,7 @@
         <v>0</v>
       </c>
       <c r="O265" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P265" s="0" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 13/10/2026 15:43 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46308.35485375</v>
+        <v>46308.655081122684</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -42461,7 +42461,7 @@
         <v>2656</v>
       </c>
       <c r="O562" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P562" s="0" t="s">
         <v>52</v>
@@ -55470,7 +55470,7 @@
         <v>2</v>
       </c>
       <c r="O825" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P825" s="0" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 15/10/2026 09:39 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -20,7 +20,7 @@
     <t>Usuário Geração:</t>
   </si>
   <si>
-    <t>Jadson Rubens Rocha de Oliveira</t>
+    <t>GABRIELLE MENDES DE ANDRADE</t>
   </si>
   <si>
     <t>Tipo Equipamento</t>
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46310.39905511574</v>
+        <v>46310.402224861115</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 15/10/2026 15:01 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46310.402224861115</v>
+        <v>46310.62601244213</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -60247,7 +60247,7 @@
         <v>4087</v>
       </c>
       <c r="O926" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="R926" s="0" t="s">
         <v>4088</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 19/10/2026 08:07 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -20,7 +20,7 @@
     <t>Usuário Geração:</t>
   </si>
   <si>
-    <t>GABRIELLE MENDES DE ANDRADE</t>
+    <t>Jadson Rubens Rocha de Oliveira</t>
   </si>
   <si>
     <t>Tipo Equipamento</t>
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46311.62599112269</v>
+        <v>46314.33837157407</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -24916,7 +24916,7 @@
         <v>0</v>
       </c>
       <c r="O221" s="0" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="P221" s="0" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 20/10/2026 08:38 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -20,7 +20,7 @@
     <t>Usuário Geração:</t>
   </si>
   <si>
-    <t>Jadson Rubens Rocha de Oliveira</t>
+    <t>GABRIELLE MENDES DE ANDRADE</t>
   </si>
   <si>
     <t>Tipo Equipamento</t>
@@ -13004,7 +13004,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46314.62219799768</v>
+        <v>46315.35998353009</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Atualiza dados — extração 23/10/2026 08:58 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4274" uniqueCount="4274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4279" uniqueCount="4279">
   <si>
     <t>Geração:</t>
   </si>
@@ -12834,6 +12834,21 @@
   </si>
   <si>
     <t>00753284812</t>
+  </si>
+  <si>
+    <t>SR /GUERRA AG BS</t>
+  </si>
+  <si>
+    <t>GUERRA AG BS</t>
+  </si>
+  <si>
+    <t>9AA02083G8C079438</t>
+  </si>
+  <si>
+    <t>00982449780</t>
+  </si>
+  <si>
+    <t>ITUPIRANGA</t>
   </si>
 </sst>
 </file>
@@ -12996,7 +13011,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W971"/>
+  <dimension ref="A1:W972"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="16384" width="9.140625" customWidth="1"/>
@@ -13007,7 +13022,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46317.66587892361</v>
+        <v>46318.37390993055</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -62381,6 +62396,50 @@
       </c>
       <c r="O971" s="0" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" s="0" t="s">
+        <v>3567</v>
+      </c>
+      <c r="B972" s="10">
+        <v>46317.68723200232</v>
+      </c>
+      <c r="C972" s="0" t="s">
+        <v>2663</v>
+      </c>
+      <c r="D972" s="0" t="s">
+        <v>2670</v>
+      </c>
+      <c r="E972" s="0" t="s">
+        <v>4274</v>
+      </c>
+      <c r="F972" s="0" t="s">
+        <v>4275</v>
+      </c>
+      <c r="G972" s="0" t="s">
+        <v>2663</v>
+      </c>
+      <c r="H972" s="0" t="s">
+        <v>4276</v>
+      </c>
+      <c r="I972" s="0" t="s">
+        <v>4277</v>
+      </c>
+      <c r="J972" s="0" t="s">
+        <v>535</v>
+      </c>
+      <c r="K972" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="L972" s="0" t="s">
+        <v>4278</v>
+      </c>
+      <c r="O972" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="V972" s="0" t="s">
+        <v>2669</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza dados — extração 26/10/2026 09:17 (via painel)
</commit_message>
<xml_diff>
--- a/dados/equipamentos.xlsx
+++ b/dados/equipamentos.xlsx
@@ -13022,7 +13022,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3">
-        <v>46318.664278414355</v>
+        <v>46321.387184444444</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -34943,7 +34943,7 @@
         <v>115</v>
       </c>
       <c r="O406" s="0" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="P406" s="0" t="s">
         <v>1945</v>

</xml_diff>